<commit_message>
Guides d'entretien FPPN : ajout de la colonne d'explication des termes et réponses attendues
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_Guides_entretiens_actuariat_20261016.xlsx
+++ b/FPPN_Guides_entretiens_actuariat_20261016.xlsx
@@ -737,7 +737,8 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Fabrice Kebe-Mambo, Ruth Miensa</t>
+          <t>Fabrice Kebe-Mambo
+Ruth Miensa</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -777,7 +778,8 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Marlène Mody, Williams Koffi</t>
+          <t>Marlène Mody
+Williams Koffi</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -817,7 +819,10 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Inès Kwekam, Issa Bamba, Ruth Miensa, Marlène Mody</t>
+          <t>Inès Kwekam, 
+Issa Bamba, 
+Ruth Miensa, 
+Marlène Mody</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -857,7 +862,8 @@
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>Ruth Miensa, Jean-Noël Sialou</t>
+          <t>Ruth Miensa,
+Jean-Noël Sialou</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr">
@@ -897,7 +903,8 @@
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>Issa Bamba, Jean-Noël Sialou</t>
+          <t>Issa Bamba, 
+Jean-Noël Sialou</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr">
@@ -937,7 +944,8 @@
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>Issa Bamba, Jean-Noël Sialou</t>
+          <t>Issa Bamba, 
+Jean-Noël Sialou</t>
         </is>
       </c>
       <c r="H14" s="10" t="inlineStr">
@@ -977,7 +985,8 @@
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>Marlène Mody, Jean-Noël Sialou</t>
+          <t>Marlène Mody, 
+Jean-Noël Sialou</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
@@ -1066,17 +1075,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:H44"/>
+  <dimension ref="B2:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1093,17 +1103,17 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="45" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Introduction : « Bonjour, je suis Jean-Noël Sialou, actuaire de l'équipe Adenka. Je travaille sur les engagements du FPPN envers les mutualistes, les provisions et les placements. Cet entretien m'aide à comprendre les prestations servies, leurs délais de paiement et les données disponibles. »</t>
+          <t>Introduction : « Bonjour, je suis Jean-Noël Sialou, Consultant Actuaire de l'équipe Adenka. Sur cette mission, je travaillerai sur les engagements du FPPN envers les mutualistes, les provisions et les placements. Cet entretien a pour but de m'aider à comprendre les prestations servies, leurs délais de paiement et les données disponibles. »</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usage interne : la colonne « À quoi elle sert » est réservée à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
+          <t>Usage interne : les colonnes « À quoi elle sert » et « Explication » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
         </is>
       </c>
     </row>
@@ -1130,15 +1140,20 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
+          <t>Explication et réponses attendues (usage interne)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
           <t>Document à demander</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1155,9 +1170,10 @@
       <c r="E8" s="15" t="n"/>
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
-      <c r="H8" s="16" t="n"/>
-    </row>
-    <row r="9" ht="32" customHeight="1">
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="16" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
       <c r="B9" s="5" t="n">
         <v>1</v>
       </c>
@@ -1178,17 +1194,22 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
+          <t>Prestation = somme ou service versé par le FPPN. Attendu : allocation décès, aide invalidité, soins, épargne de fin de carrière, aides sociales. Note chaque prestation citée.</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
           <t>Liste des prestations et barèmes</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
       <c r="B10" s="5" t="n">
         <v>2</v>
       </c>
@@ -1209,17 +1230,22 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
+          <t>Barème = grille de montants (fixe, ou selon le grade ou l'ancienneté). Ayants droit = conjoint et enfants. Attendu : montant fixe ou plafonné. Alerte : « au cas par cas ».</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
           <t>Règlement des prestations</t>
         </is>
       </c>
-      <c r="G10" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="32" customHeight="1">
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="46" customHeight="1">
       <c r="B11" s="5" t="n">
         <v>3</v>
       </c>
@@ -1240,17 +1266,22 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
+          <t>Attendu : « non », ou des dates de changement avec une décision du conseil ou de l'AG. Alerte : changement sans décision écrite.</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
           <t>Décisions du conseil ou de l'AG</t>
         </is>
       </c>
-      <c r="G11" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12" ht="32" customHeight="1">
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12" ht="46" customHeight="1">
       <c r="B12" s="5" t="n">
         <v>4</v>
       </c>
@@ -1269,15 +1300,20 @@
           <t>Une rente crée un engagement sur plusieurs années, à provisionner autrement.</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13" ht="32" customHeight="1">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Capital = paiement unique. Rente = paiement régulier pendant plusieurs années. Si rente : demande la durée et les bénéficiaires.</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="46" customHeight="1">
       <c r="B13" s="5" t="n">
         <v>5</v>
       </c>
@@ -1296,15 +1332,20 @@
           <t>Identifier les engagements longs envers les retraités.</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr"/>
-      <c r="G13" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14" ht="32" customHeight="1">
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : oui pour la santé ou le décès, avec ou sans cotisation. Alerte : couverture à vie sans cotisation, donc engagement lourd non financé.</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14" ht="46" customHeight="1">
       <c r="B14" s="5" t="n">
         <v>6</v>
       </c>
@@ -1325,17 +1366,22 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
+          <t>CGRAE = caisse de retraite des fonctionnaires. Attendu : un partage des frais de soins des retraités entre la CGRAE et le FPPN. Demande la convention.</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
           <t>Convention avec la CGRAE</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr"/>
-    </row>
-    <row r="15" ht="32" customHeight="1">
+      <c r="I14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15" ht="46" customHeight="1">
       <c r="B15" s="5" t="n">
         <v>7</v>
       </c>
@@ -1354,13 +1400,18 @@
           <t>Préciser qui est couvert à une date donnée.</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr"/>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Délai de carence = période après l'adhésion sans droit aux prestations. Attendu : aucun, ou un nombre de mois de cotisation.</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="B16" s="14" t="inlineStr">
@@ -1373,9 +1424,10 @@
       <c r="E16" s="15" t="n"/>
       <c r="F16" s="15" t="n"/>
       <c r="G16" s="15" t="n"/>
-      <c r="H16" s="16" t="n"/>
-    </row>
-    <row r="17" ht="32" customHeight="1">
+      <c r="H16" s="15" t="n"/>
+      <c r="I16" s="16" t="n"/>
+    </row>
+    <row r="17" ht="46" customHeight="1">
       <c r="B17" s="5" t="n">
         <v>8</v>
       </c>
@@ -1396,17 +1448,22 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
+          <t>Attendu : déclaration, dossier, vérification, validation, paiement. Repère les dates enregistrées à chaque étape.</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
           <t>Procédure de traitement</t>
         </is>
       </c>
-      <c r="G17" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr"/>
-    </row>
-    <row r="18" ht="32" customHeight="1">
+      <c r="H17" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18" ht="46" customHeight="1">
       <c r="B18" s="5" t="n">
         <v>9</v>
       </c>
@@ -1425,15 +1482,20 @@
           <t>Estimer les prestations survenues mais pas encore payées à la clôture.</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr"/>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : un délai en semaines ou en mois. Plus il est long, plus la provision pour dossiers en cours doit être élevée.</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19" ht="46" customHeight="1">
       <c r="B19" s="5" t="n">
         <v>10</v>
       </c>
@@ -1452,15 +1514,20 @@
           <t>Estimer les dossiers survenus mais pas encore déclarés (tardifs).</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr"/>
-      <c r="G19" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20" ht="32" customHeight="1">
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Tardif = événement survenu avant la clôture mais déclaré après. Attendu : un délai fixé par les règles, ou aucun. Alerte : déclarations plusieurs années après.</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20" ht="46" customHeight="1">
       <c r="B20" s="5" t="n">
         <v>11</v>
       </c>
@@ -1481,17 +1548,22 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
+          <t>Stock = dossiers reçus ou acceptés mais non payés. Attendu : un nombre et un montant. Alerte : « on ne sait pas », donc pas de suivi.</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
           <t>Liste des dossiers en attente</t>
         </is>
       </c>
-      <c r="G20" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21" ht="32" customHeight="1">
+      <c r="H20" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21" ht="46" customHeight="1">
       <c r="B21" s="5" t="n">
         <v>12</v>
       </c>
@@ -1510,15 +1582,20 @@
           <t>Repérer des tensions de trésorerie ou des provisions insuffisantes.</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr"/>
-      <c r="G21" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr"/>
-    </row>
-    <row r="22" ht="32" customHeight="1">
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : oui ou non, avec la cause (trésorerie, dossiers incomplets, cotisations non reversées). Alerte : retards répétés.</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr"/>
+      <c r="H21" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22" ht="60" customHeight="1">
       <c r="B22" s="5" t="n">
         <v>13</v>
       </c>
@@ -1539,15 +1616,20 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
+          <t>Arriérés = dettes anciennes envers mutualistes et prestataires. Attendu : elles étaient au bilan en dettes ou provisions. Alerte : dettes payées sans avoir été enregistrées.</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
           <t>État des arriérés apurés</t>
         </is>
       </c>
-      <c r="G22" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr"/>
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="B23" s="14" t="inlineStr">
@@ -1560,9 +1642,10 @@
       <c r="E23" s="15" t="n"/>
       <c r="F23" s="15" t="n"/>
       <c r="G23" s="15" t="n"/>
-      <c r="H23" s="16" t="n"/>
-    </row>
-    <row r="24" ht="32" customHeight="1">
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="16" t="n"/>
+    </row>
+    <row r="24" ht="46" customHeight="1">
       <c r="B24" s="5" t="n">
         <v>14</v>
       </c>
@@ -1583,17 +1666,22 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
+          <t>Tiers payant = le FPPN paie directement la clinique. Remboursement = le mutualiste avance puis est remboursé. Attendu : l'un, l'autre ou les deux.</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
           <t>Conventions avec les prestataires</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25" ht="32" customHeight="1">
+      <c r="I24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25" ht="46" customHeight="1">
       <c r="B25" s="5" t="n">
         <v>15</v>
       </c>
@@ -1612,15 +1700,20 @@
           <t>Estimer les soins réalisés mais pas encore facturés à la clôture.</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr"/>
-      <c r="G25" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26" ht="32" customHeight="1">
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : un délai en semaines ou en mois. Plus il est long, plus il reste de soins non facturés à la clôture.</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr"/>
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26" ht="46" customHeight="1">
       <c r="B26" s="5" t="n">
         <v>16</v>
       </c>
@@ -1639,13 +1732,18 @@
           <t>Éviter d'oublier ou de compter deux fois une partie du coût santé.</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr"/>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : oui (facture interne) ou non (coût dans les charges du centre). Note la réponse pour ne pas compter deux fois le coût.</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr"/>
+      <c r="I26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="B27" s="14" t="inlineStr">
@@ -1658,9 +1756,10 @@
       <c r="E27" s="15" t="n"/>
       <c r="F27" s="15" t="n"/>
       <c r="G27" s="15" t="n"/>
-      <c r="H27" s="16" t="n"/>
-    </row>
-    <row r="28" ht="32" customHeight="1">
+      <c r="H27" s="15" t="n"/>
+      <c r="I27" s="16" t="n"/>
+    </row>
+    <row r="28" ht="46" customHeight="1">
       <c r="B28" s="5" t="n">
         <v>17</v>
       </c>
@@ -1679,13 +1778,18 @@
           <t>Savoir si les données peuvent être extraites facilement.</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr"/>
-      <c r="G28" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr"/>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : nom d'un logiciel, fichiers Excel ou registres papier. Papier = extraction longue, prévoir plus de temps.</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr"/>
+      <c r="H28" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr"/>
     </row>
     <row r="29" ht="46" customHeight="1">
       <c r="B29" s="5" t="n">
@@ -1708,15 +1812,20 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
+          <t>Les 3 dates sont essentielles. Attendu : oui, ou seulement la date de paiement. Si une date manque, demande où elle est conservée.</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
           <t>Fichier des prestations payées (Excel)</t>
         </is>
       </c>
-      <c r="G29" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr"/>
+      <c r="H29" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr"/>
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="B30" s="5" t="n">
@@ -1737,13 +1846,18 @@
           <t>Pouvoir relier les prestations au fichier des mutualistes.</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr"/>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Matricule = identifiant unique du policier. Attendu : oui. Alerte : nom seul, risque de doublons.</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr"/>
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr"/>
+      <c r="I30" s="6" t="inlineStr"/>
     </row>
     <row r="31" ht="32" customHeight="1">
       <c r="B31" s="5" t="n">
@@ -1766,15 +1880,20 @@
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
+          <t>Attendu : tableaux par mois ou par année. S'ils existent, ils servent à contrôler les fichiers reçus.</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
           <t>Tableaux de bord des prestations</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr"/>
+      <c r="I31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="B32" s="14" t="inlineStr">
@@ -1787,7 +1906,8 @@
       <c r="E32" s="15" t="n"/>
       <c r="F32" s="15" t="n"/>
       <c r="G32" s="15" t="n"/>
-      <c r="H32" s="16" t="n"/>
+      <c r="H32" s="15" t="n"/>
+      <c r="I32" s="16" t="n"/>
     </row>
     <row r="33" ht="32" customHeight="1">
       <c r="B33" s="5" t="n">
@@ -1808,15 +1928,20 @@
           <t>Apprécier la fiabilité des montants payés.</t>
         </is>
       </c>
-      <c r="F33" s="6" t="inlineStr"/>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : un agent prépare, un responsable valide. Alerte : une seule personne fait tout.</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr"/>
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr"/>
-    </row>
-    <row r="34" ht="32" customHeight="1">
+      <c r="I33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34" ht="46" customHeight="1">
       <c r="B34" s="5" t="n">
         <v>22</v>
       </c>
@@ -1835,13 +1960,18 @@
           <t>Repérer les risques de doublons dans les données.</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr"/>
-      <c r="G34" s="6" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Doublon = même prestation payée deux fois. Attendu : contrôle dans le logiciel ou un registre. Alerte : aucun contrôle.</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr"/>
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H34" s="6" t="inlineStr"/>
+      <c r="I34" s="6" t="inlineStr"/>
     </row>
     <row r="35" ht="32" customHeight="1">
       <c r="B35" s="5" t="n">
@@ -1862,13 +1992,18 @@
           <t>Apprécier la traçabilité des paiements.</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr"/>
-      <c r="G35" s="6" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : surtout par virement. Alerte : espèces fréquentes, traçabilité faible.</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr"/>
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H35" s="6" t="inlineStr"/>
+      <c r="I35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="B36" s="14" t="inlineStr">
@@ -1881,9 +2016,10 @@
       <c r="E36" s="15" t="n"/>
       <c r="F36" s="15" t="n"/>
       <c r="G36" s="15" t="n"/>
-      <c r="H36" s="16" t="n"/>
-    </row>
-    <row r="37" ht="32" customHeight="1">
+      <c r="H36" s="15" t="n"/>
+      <c r="I36" s="16" t="n"/>
+    </row>
+    <row r="37" ht="46" customHeight="1">
       <c r="B37" s="5" t="n">
         <v>24</v>
       </c>
@@ -1904,17 +2040,22 @@
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
+          <t>Litige = désaccord en réclamation ou en justice. Attendu : un nombre et des montants. S'il y en a, une provision peut être nécessaire.</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
           <t>État des litiges</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr"/>
-    </row>
-    <row r="38" ht="32" customHeight="1">
+      <c r="I37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38" ht="46" customHeight="1">
       <c r="B38" s="5" t="n">
         <v>25</v>
       </c>
@@ -1933,13 +2074,18 @@
           <t>Vérifier le lien entre les dossiers et les provisions au bilan.</t>
         </is>
       </c>
-      <c r="F38" s="6" t="inlineStr"/>
-      <c r="G38" s="6" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : la liste des dossiers en attente transmise à la comptabilité à la clôture. Alerte : aucune transmission, donc dettes absentes du bilan.</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr"/>
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H38" s="6" t="inlineStr"/>
+      <c r="I38" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="B40" s="2" t="inlineStr">
@@ -1978,21 +2124,21 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B36:H36"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B32:H32"/>
-    <mergeCell ref="B27:H27"/>
-    <mergeCell ref="B41:H41"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B44:H44"/>
-    <mergeCell ref="B43:H43"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B42:H42"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="B16:I16"/>
+    <mergeCell ref="B42:I42"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B32:I32"/>
+    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B43:I43"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G8:G39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H8:H39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2008,17 +2154,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:H41"/>
+  <dimension ref="B2:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -2035,17 +2182,17 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="45" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Introduction : « Bonjour, je suis Jean-Noël Sialou, actuaire de l'équipe Adenka. Je travaille sur les engagements du FPPN envers les mutualistes, les provisions et les placements. Cet entretien m'aide à comprendre comment les provisions sont calculées et suivies. »</t>
+          <t>Introduction : « Bonjour, je suis Jean-Noël Sialou, Consultant Actuaire de l'équipe Adenka. Sur cette mission, je travaillerai sur les engagements du FPPN envers les mutualistes, les provisions et les placements. Cet entretien a pour but de m'aider à comprendre comment les provisions sont calculées et suivies. »</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usage interne : la colonne « À quoi elle sert » est réservée à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
+          <t>Usage interne : les colonnes « À quoi elle sert » et « Explication » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
         </is>
       </c>
     </row>
@@ -2072,15 +2219,20 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
+          <t>Explication et réponses attendues (usage interne)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
           <t>Document à demander</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2097,9 +2249,10 @@
       <c r="E8" s="15" t="n"/>
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
-      <c r="H8" s="16" t="n"/>
-    </row>
-    <row r="9" ht="32" customHeight="1">
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="16" t="n"/>
+    </row>
+    <row r="9" ht="46" customHeight="1">
       <c r="B9" s="5" t="n">
         <v>1</v>
       </c>
@@ -2120,17 +2273,22 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
+          <t>Provision = montant inscrit au bilan pour une dette future. Attendu : prestations à payer, épargne, risques, créances douteuses. Alerte : « aucune ».</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
           <t>Détail des provisions par nature</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="46" customHeight="1">
       <c r="B10" s="5" t="n">
         <v>2</v>
       </c>
@@ -2151,15 +2309,20 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
+          <t>Attendu : liste des dossiers connus, pourcentage des cotisations, forfait ou calcul actuariel. Le plus fiable : dossiers connus plus estimation des tardifs.</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
           <t>Note ou fichier de calcul</t>
         </is>
       </c>
-      <c r="G10" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr"/>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="B11" s="5" t="n">
@@ -2180,13 +2343,18 @@
           <t>Savoir à qui poser les questions techniques de suivi.</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr"/>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : le comptable ou le DAF calcule, le DG ou le conseil valide.</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="B12" s="5" t="n">
@@ -2207,15 +2375,20 @@
           <t>Expliquer les variations d'une année à l'autre.</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13" ht="32" customHeight="1">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : non, ou un changement daté et expliqué. Alerte : changement sans explication.</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="60" customHeight="1">
       <c r="B13" s="5" t="n">
         <v>5</v>
       </c>
@@ -2234,15 +2407,20 @@
           <t>Vérifier qu'une partie des engagements n'est pas oubliée.</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr"/>
-      <c r="G13" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14" ht="32" customHeight="1">
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Survenus non déclarés (IBNR) = événements arrivés avant la clôture, encore inconnus. Attendu : souvent « non ». Dans ce cas, les provisions sont probablement trop faibles.</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14" ht="46" customHeight="1">
       <c r="B14" s="5" t="n">
         <v>6</v>
       </c>
@@ -2261,15 +2439,20 @@
           <t>Les engagements longs sont souvent absents des comptes.</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr"/>
-      <c r="G14" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr"/>
-    </row>
-    <row r="15" ht="18" customHeight="1">
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Engagement long = promesse sur plusieurs années, par exemple les soins des retraités à vie. Attendu : souvent « non ». Point important pour ton rapport.</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15" ht="32" customHeight="1">
       <c r="B15" s="5" t="n">
         <v>7</v>
       </c>
@@ -2290,17 +2473,22 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
+          <t>Attendu : le plus souvent non, sinon le nom du cabinet et l'année. Demande le rapport.</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
           <t>Rapport actuariel existant</t>
         </is>
       </c>
-      <c r="G15" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr"/>
-    </row>
-    <row r="16" ht="32" customHeight="1">
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
       <c r="B16" s="5" t="n">
         <v>8</v>
       </c>
@@ -2319,13 +2507,18 @@
           <t>Comparer les hypothèses à celles que je retiendrai.</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr"/>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Table de mortalité = probabilité de décès par âge (CIMA H par exemple). Taux d'actualisation = taux pour ramener un montant futur à aujourd'hui. Attendu : souvent aucune hypothèse.</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="B17" s="14" t="inlineStr">
@@ -2338,9 +2531,10 @@
       <c r="E17" s="15" t="n"/>
       <c r="F17" s="15" t="n"/>
       <c r="G17" s="15" t="n"/>
-      <c r="H17" s="16" t="n"/>
-    </row>
-    <row r="18" ht="32" customHeight="1">
+      <c r="H17" s="15" t="n"/>
+      <c r="I17" s="16" t="n"/>
+    </row>
+    <row r="18" ht="46" customHeight="1">
       <c r="B18" s="5" t="n">
         <v>9</v>
       </c>
@@ -2359,13 +2553,18 @@
           <t>Tester si les provisions passées étaient suffisantes.</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr"/>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Boni = provision supérieure aux paiements réels. Mali = provision inférieure. Attendu : souvent pas de suivi. S'il existe, demande le tableau.</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr"/>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="B19" s="5" t="n">
@@ -2386,15 +2585,20 @@
           <t>Repérer les années à examiner en priorité.</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr"/>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : non, ou des années citées avec une cause. Note ces années pour les examiner en priorité.</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20" ht="32" customHeight="1">
+      <c r="I19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20" ht="46" customHeight="1">
       <c r="B20" s="5" t="n">
         <v>11</v>
       </c>
@@ -2413,15 +2617,20 @@
           <t>Savoir quelles règles de provisionnement s'appliquent.</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr"/>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Référentiel = ensemble des règles comptables. Attendu : PCMS (plan comptable des mutuelles sociales) ou SYSCOHADA. Note l'année d'un éventuel changement.</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21" ht="32" customHeight="1">
+      <c r="I20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21" ht="46" customHeight="1">
       <c r="B21" s="5" t="n">
         <v>12</v>
       </c>
@@ -2442,15 +2651,20 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
+          <t>AIRMS = régulateur des mutuelles sociales. Attendu : un ratio de réserves ou de couverture. Note le ratio demandé et le niveau atteint.</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
           <t>Courriers de l'AIRMS</t>
         </is>
       </c>
-      <c r="G21" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr"/>
+      <c r="H21" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr"/>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="B22" s="5" t="n">
@@ -2473,15 +2687,20 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
+          <t>Attendu : non, ou des courriers, mises en demeure, plan de redressement. Demande les courriers.</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
           <t>Rapports de contrôle de l'AIRMS</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr"/>
+      <c r="I22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="B23" s="14" t="inlineStr">
@@ -2494,9 +2713,10 @@
       <c r="E23" s="15" t="n"/>
       <c r="F23" s="15" t="n"/>
       <c r="G23" s="15" t="n"/>
-      <c r="H23" s="16" t="n"/>
-    </row>
-    <row r="24" ht="32" customHeight="1">
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="16" t="n"/>
+    </row>
+    <row r="24" ht="46" customHeight="1">
       <c r="B24" s="5" t="n">
         <v>14</v>
       </c>
@@ -2517,17 +2737,22 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
+          <t>Attendu : épargne de fin de carrière, Plan Épargne Plus, ou aucun. Si aucun, les questions sur l'épargne tombent.</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
           <t>Description des produits d'épargne</t>
         </is>
       </c>
-      <c r="G24" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25" ht="32" customHeight="1">
+      <c r="H24" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25" ht="60" customHeight="1">
       <c r="B25" s="5" t="n">
         <v>15</v>
       </c>
@@ -2548,17 +2773,22 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
+          <t>Taux servi = intérêt crédité aux épargnants. Garanti = promis à l'avance. Attendu : taux fixe ou décidé chaque année. Alerte : taux supérieur au rendement des placements.</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
           <t>Décisions fixant le taux</t>
         </is>
       </c>
-      <c r="G25" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26" ht="32" customHeight="1">
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26" ht="46" customHeight="1">
       <c r="B26" s="5" t="n">
         <v>16</v>
       </c>
@@ -2579,15 +2809,20 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
+          <t>Rapprochement = vérifier que la somme des comptes individuels égale le chiffre du bilan. Attendu : oui, avec un tableau. Alerte : écart non expliqué.</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
           <t>Rapprochement comptes individuels et bilan</t>
         </is>
       </c>
-      <c r="G26" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr"/>
+      <c r="H26" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="B27" s="14" t="inlineStr">
@@ -2600,9 +2835,10 @@
       <c r="E27" s="15" t="n"/>
       <c r="F27" s="15" t="n"/>
       <c r="G27" s="15" t="n"/>
-      <c r="H27" s="16" t="n"/>
-    </row>
-    <row r="28" ht="32" customHeight="1">
+      <c r="H27" s="15" t="n"/>
+      <c r="I27" s="16" t="n"/>
+    </row>
+    <row r="28" ht="60" customHeight="1">
       <c r="B28" s="5" t="n">
         <v>17</v>
       </c>
@@ -2621,13 +2857,18 @@
           <t>Planifier mes calculs à cette date.</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr"/>
-      <c r="G28" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr"/>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Situation au 31/08/2026 = comptes arrêtés en cours d'année, ce n'est pas une clôture annuelle. Attendu : une date. Alerte : provisions non recalculées à cette date.</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr"/>
+      <c r="H28" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr"/>
     </row>
     <row r="29" ht="32" customHeight="1">
       <c r="B29" s="5" t="n">
@@ -2650,15 +2891,20 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
+          <t>Attendu : des fichiers Excel par année. Alerte : calculs non conservés.</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
           <t>Fichiers de calcul 2019 à 2026</t>
         </is>
       </c>
-      <c r="G29" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr"/>
+      <c r="H29" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="B30" s="14" t="inlineStr">
@@ -2671,7 +2917,8 @@
       <c r="E30" s="15" t="n"/>
       <c r="F30" s="15" t="n"/>
       <c r="G30" s="15" t="n"/>
-      <c r="H30" s="16" t="n"/>
+      <c r="H30" s="15" t="n"/>
+      <c r="I30" s="16" t="n"/>
     </row>
     <row r="31" ht="32" customHeight="1">
       <c r="B31" s="5" t="n">
@@ -2692,13 +2939,18 @@
           <t>Apprécier la fiabilité des montants au bilan.</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr"/>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : oui, par le DAF ou le chef comptable. Alerte : aucune revue.</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr"/>
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr"/>
+      <c r="I31" s="6" t="inlineStr"/>
     </row>
     <row r="32" ht="32" customHeight="1">
       <c r="B32" s="5" t="n">
@@ -2719,13 +2971,18 @@
           <t>Identifier le niveau de validation.</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr"/>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : le DAF puis le DG, parfois le conseil. Note qui signe.</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr"/>
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr"/>
+      <c r="I32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="B33" s="14" t="inlineStr">
@@ -2738,9 +2995,10 @@
       <c r="E33" s="15" t="n"/>
       <c r="F33" s="15" t="n"/>
       <c r="G33" s="15" t="n"/>
-      <c r="H33" s="16" t="n"/>
-    </row>
-    <row r="34" ht="32" customHeight="1">
+      <c r="H33" s="15" t="n"/>
+      <c r="I33" s="16" t="n"/>
+    </row>
+    <row r="34" ht="46" customHeight="1">
       <c r="B34" s="5" t="n">
         <v>21</v>
       </c>
@@ -2759,13 +3017,18 @@
           <t>Rapprocher cotisations et engagements par garantie.</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr"/>
-      <c r="G34" s="6" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : non, la cotisation est globale ; ou une clé de répartition par garantie. Si non, la répartition devra être estimée.</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr"/>
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H34" s="6" t="inlineStr"/>
+      <c r="I34" s="6" t="inlineStr"/>
     </row>
     <row r="35" ht="32" customHeight="1">
       <c r="B35" s="5" t="n">
@@ -2786,13 +3049,18 @@
           <t>Préparer l'analyse actifs / passifs.</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr"/>
-      <c r="G35" s="6" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : le plus souvent non. Si oui, note lesquels : ils servent directement à l'adossement.</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr"/>
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H35" s="6" t="inlineStr"/>
+      <c r="I35" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="B37" s="2" t="inlineStr">
@@ -2831,21 +3099,21 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B27:H27"/>
-    <mergeCell ref="B40:H40"/>
-    <mergeCell ref="B41:H41"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B39:H39"/>
-    <mergeCell ref="B30:H30"/>
-    <mergeCell ref="B38:H38"/>
-    <mergeCell ref="B33:H33"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B39:I39"/>
+    <mergeCell ref="B38:I38"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B17:I17"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G8:G36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H8:H36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2861,17 +3129,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:H37"/>
+  <dimension ref="B2:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -2888,17 +3157,17 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="45" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Introduction : « Bonjour, je suis Jean-Noël Sialou, actuaire de l'équipe Adenka. Je travaille sur les engagements du FPPN envers les mutualistes, les provisions et les placements. Cet entretien m'aide à comprendre les placements et leur capacité à couvrir les engagements. »</t>
+          <t>Introduction : « Bonjour, je suis Jean-Noël Sialou, Consultant Actuaire de l'équipe Adenka. Sur cette mission, je travaillerai sur les engagements du FPPN envers les mutualistes, les provisions et les placements. Cet entretien a pour but de m'aider à comprendre les placements et leur capacité à couvrir les engagements. »</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usage interne : la colonne « À quoi elle sert » est réservée à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
+          <t>Usage interne : les colonnes « À quoi elle sert » et « Explication » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
         </is>
       </c>
     </row>
@@ -2925,15 +3194,20 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
+          <t>Explication et réponses attendues (usage interne)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
           <t>Document à demander</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2950,9 +3224,10 @@
       <c r="E8" s="15" t="n"/>
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
-      <c r="H8" s="16" t="n"/>
-    </row>
-    <row r="9" ht="32" customHeight="1">
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="16" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
       <c r="B9" s="5" t="n">
         <v>1</v>
       </c>
@@ -2973,17 +3248,22 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
+          <t>Dépôt à terme = argent bloqué en banque pour une durée fixe. Obligation = prêt à un État ou une entreprise. Attendu : surtout des dépôts à terme et des comptes bancaires.</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
           <t>Inventaire des placements</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="46" customHeight="1">
       <c r="B10" s="5" t="n">
         <v>2</v>
       </c>
@@ -3002,15 +3282,20 @@
           <t>Mesurer la dépendance à un seul établissement.</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="32" customHeight="1">
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Émetteur = celui qui émet le titre (État, entreprise). Alerte : une grande partie des placements dans une seule banque.</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="46" customHeight="1">
       <c r="B11" s="5" t="n">
         <v>3</v>
       </c>
@@ -3031,15 +3316,20 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
+          <t>Échéance = date de remboursement du placement. Attendu : une liste de dates. Compare-les aux dates de paiement de l'épargne et des prestations.</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
           <t>Échéancier des placements</t>
         </is>
       </c>
-      <c r="G11" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr"/>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="B12" s="5" t="n">
@@ -3060,15 +3350,20 @@
           <t>Savoir quels actifs sont réellement disponibles en cas de besoin.</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13" ht="32" customHeight="1">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : oui avec perte d'intérêts, ou non. Alerte : fonds bloqués alors que des paiements sont en retard.</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="46" customHeight="1">
       <c r="B13" s="5" t="n">
         <v>5</v>
       </c>
@@ -3087,13 +3382,18 @@
           <t>Comparer le rendement au taux servi sur l'épargne.</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr"/>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Rendement = intérêts reçus ÷ montant placé. Attendu : un taux par année. Compare-le au taux servi sur l'épargne.</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="14" t="inlineStr">
@@ -3106,7 +3406,8 @@
       <c r="E14" s="15" t="n"/>
       <c r="F14" s="15" t="n"/>
       <c r="G14" s="15" t="n"/>
-      <c r="H14" s="16" t="n"/>
+      <c r="H14" s="15" t="n"/>
+      <c r="I14" s="16" t="n"/>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="B15" s="5" t="n">
@@ -3129,17 +3430,22 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
+          <t>Attendu : un document validé par le conseil, ou des décisions au cas par cas du DG. Alerte : aucune règle.</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
           <t>Politique de placement</t>
         </is>
       </c>
-      <c r="G15" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr"/>
-    </row>
-    <row r="16" ht="32" customHeight="1">
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16" ht="46" customHeight="1">
       <c r="B16" s="5" t="n">
         <v>7</v>
       </c>
@@ -3158,15 +3464,20 @@
           <t>Apprécier l'adossement entre actifs et engagements.</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr"/>
-      <c r="G16" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr"/>
-    </row>
-    <row r="17" ht="32" customHeight="1">
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Adossement = faire correspondre les dates d'échéance des placements aux dates de paiement. Attendu : souvent « non ». Dans ce cas : risque de manque de liquidités.</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17" ht="46" customHeight="1">
       <c r="B17" s="5" t="n">
         <v>8</v>
       </c>
@@ -3185,13 +3496,18 @@
           <t>Vérifier la conformité du portefeuille.</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr"/>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : des règles de l'AIRMS sur les types d'actifs ou les limites par banque, ou « pas à ma connaissance ».</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="B18" s="14" t="inlineStr">
@@ -3204,7 +3520,8 @@
       <c r="E18" s="15" t="n"/>
       <c r="F18" s="15" t="n"/>
       <c r="G18" s="15" t="n"/>
-      <c r="H18" s="16" t="n"/>
+      <c r="H18" s="15" t="n"/>
+      <c r="I18" s="16" t="n"/>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="B19" s="5" t="n">
@@ -3227,15 +3544,20 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
+          <t>Attendu : plan de trésorerie mensuel ou suivi au jour le jour. Alerte : aucune prévision.</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
           <t>Prévisions de trésorerie</t>
         </is>
       </c>
-      <c r="G19" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr"/>
+      <c r="H19" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr"/>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="B20" s="5" t="n">
@@ -3256,13 +3578,18 @@
           <t>Repérer les périodes de tension.</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr"/>
-      <c r="G20" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : non, ou des périodes précises, souvent liées aux cotisations non reversées. Note les dates.</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="B21" s="14" t="inlineStr">
@@ -3275,9 +3602,10 @@
       <c r="E21" s="15" t="n"/>
       <c r="F21" s="15" t="n"/>
       <c r="G21" s="15" t="n"/>
-      <c r="H21" s="16" t="n"/>
-    </row>
-    <row r="22" ht="32" customHeight="1">
+      <c r="H21" s="15" t="n"/>
+      <c r="I21" s="16" t="n"/>
+    </row>
+    <row r="22" ht="46" customHeight="1">
       <c r="B22" s="5" t="n">
         <v>11</v>
       </c>
@@ -3298,17 +3626,22 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
+          <t>Créance = argent dû au FPPN. Attendu : un montant, un accord de remboursement ou des relances. Alerte : aucun recouvrement depuis longtemps.</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
           <t>État des cotisations non reversées</t>
         </is>
       </c>
-      <c r="G22" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="32" customHeight="1">
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="46" customHeight="1">
       <c r="B23" s="5" t="n">
         <v>12</v>
       </c>
@@ -3329,15 +3662,20 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
+          <t>Encours = capital restant dû par les emprunteurs. Impayé = échéance non remboursée. Attendu : un montant total et une part d'impayés.</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
           <t>Encours et impayés des prêts</t>
         </is>
       </c>
-      <c r="G23" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr"/>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr"/>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="B24" s="5" t="n">
@@ -3360,17 +3698,22 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
+          <t>Attendu : expertise récente ou valeur d'achat. Alerte : aucune évaluation depuis des années.</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
           <t>Dernière évaluation immobilière</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25" ht="32" customHeight="1">
+      <c r="I24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25" ht="46" customHeight="1">
       <c r="B25" s="5" t="n">
         <v>14</v>
       </c>
@@ -3389,13 +3732,18 @@
           <t>Savoir si cet actif génère de la trésorerie.</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr"/>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Location-vente = le locataire devient propriétaire après avoir payé tous les loyers. Attendu : oui avec un montant, ou projet pas encore livré.</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr"/>
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr"/>
+      <c r="I25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="B26" s="14" t="inlineStr">
@@ -3408,7 +3756,8 @@
       <c r="E26" s="15" t="n"/>
       <c r="F26" s="15" t="n"/>
       <c r="G26" s="15" t="n"/>
-      <c r="H26" s="16" t="n"/>
+      <c r="H26" s="15" t="n"/>
+      <c r="I26" s="16" t="n"/>
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="B27" s="5" t="n">
@@ -3429,15 +3778,20 @@
           <t>Apprécier la sécurité des placements.</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr"/>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : deux signatures (DG et DAF par exemple). Alerte : une seule signature.</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr"/>
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr"/>
-    </row>
-    <row r="28" ht="32" customHeight="1">
+      <c r="I27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28" ht="46" customHeight="1">
       <c r="B28" s="5" t="n">
         <v>16</v>
       </c>
@@ -3456,13 +3810,18 @@
           <t>Vérifier l'existence des placements.</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr"/>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Rapprochement bancaire = comparer la comptabilité aux relevés de la banque. Attendu : chaque mois, signé. Alerte : rare ou non fait.</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr"/>
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr"/>
+      <c r="I28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="B29" s="14" t="inlineStr">
@@ -3475,7 +3834,8 @@
       <c r="E29" s="15" t="n"/>
       <c r="F29" s="15" t="n"/>
       <c r="G29" s="15" t="n"/>
-      <c r="H29" s="16" t="n"/>
+      <c r="H29" s="15" t="n"/>
+      <c r="I29" s="16" t="n"/>
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="B30" s="5" t="n">
@@ -3496,15 +3856,20 @@
           <t>Mesurer l'effet de l'apurement sur les placements restants.</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr"/>
-      <c r="G30" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31" ht="32" customHeight="1">
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : trésorerie, retrait de placements, emprunt ou apport de l'État. Note la source et le montant.</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr"/>
+      <c r="H30" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31" ht="46" customHeight="1">
       <c r="B31" s="5" t="n">
         <v>18</v>
       </c>
@@ -3523,13 +3888,18 @@
           <t>Exclure les actifs non disponibles de la couverture.</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr"/>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Nanti = bloqué en garantie d'un prêt. Attendu : non. Si oui, ces placements ne peuvent pas servir à payer les mutualistes.</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr"/>
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr"/>
+      <c r="I31" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="B33" s="2" t="inlineStr">
@@ -3568,21 +3938,21 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B36:H36"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B26:H26"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B35:H35"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B29:H29"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B34:H34"/>
-    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="B18:I18"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="B37:I37"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B26:I26"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G8:G32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H8:H32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3598,17 +3968,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:H39"/>
+  <dimension ref="B2:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -3625,17 +3996,17 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="45" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Introduction : « Bonjour, je suis Jean-Noël Sialou, actuaire de l'équipe Adenka. Je travaille sur les engagements du FPPN envers les mutualistes, les provisions et les placements. Cet entretien m'aide à comprendre les cotisations, les effectifs et le fichier des mutualistes. »</t>
+          <t>Introduction : « Bonjour, je suis Jean-Noël Sialou, Consultant Actuaire de l'équipe Adenka. Sur cette mission, je travaillerai sur les engagements du FPPN envers les mutualistes, les provisions et les placements. Cet entretien a pour but de m'aider à comprendre les cotisations, les effectifs et le fichier des mutualistes. »</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usage interne : la colonne « À quoi elle sert » est réservée à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
+          <t>Usage interne : les colonnes « À quoi elle sert » et « Explication » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
         </is>
       </c>
     </row>
@@ -3662,15 +4033,20 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
+          <t>Explication et réponses attendues (usage interne)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
           <t>Document à demander</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3687,9 +4063,10 @@
       <c r="E8" s="15" t="n"/>
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
-      <c r="H8" s="16" t="n"/>
-    </row>
-    <row r="9" ht="32" customHeight="1">
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="16" t="n"/>
+    </row>
+    <row r="9" ht="46" customHeight="1">
       <c r="B9" s="5" t="n">
         <v>1</v>
       </c>
@@ -3710,17 +4087,22 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
+          <t>Catégories = actifs, retraités, autres membres. Attendu : montant fixe par mois ou pourcentage du salaire. Note les changements depuis 2020 et leur date.</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
           <t>Barème des cotisations 2020-2026</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="46" customHeight="1">
       <c r="B10" s="5" t="n">
         <v>2</v>
       </c>
@@ -3739,15 +4121,20 @@
           <t>Vérifier si chaque garantie est financée.</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="32" customHeight="1">
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Clé de répartition = part de la cotisation affectée à chaque garantie. Attendu : souvent aucune. Dans ce cas, je l'estimerai.</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="46" customHeight="1">
       <c r="B11" s="5" t="n">
         <v>3</v>
       </c>
@@ -3766,13 +4153,18 @@
           <t>Les retraités coûtent plus cher en santé ; savoir s'ils financent leur couverture.</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr"/>
-      <c r="G11" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : oui, prélevés sur la pension ou en paiement direct, ou non. Alerte : retraités couverts sans cotiser.</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="B12" s="5" t="n">
@@ -3793,13 +4185,18 @@
           <t>Savoir si l'effectif couvert est stable.</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : oui pour les policiers en activité. Si l'adhésion est facultative, l'effectif peut baisser.</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="14" t="inlineStr">
@@ -3812,9 +4209,10 @@
       <c r="E13" s="15" t="n"/>
       <c r="F13" s="15" t="n"/>
       <c r="G13" s="15" t="n"/>
-      <c r="H13" s="16" t="n"/>
-    </row>
-    <row r="14" ht="32" customHeight="1">
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="16" t="n"/>
+    </row>
+    <row r="14" ht="46" customHeight="1">
       <c r="B14" s="5" t="n">
         <v>5</v>
       </c>
@@ -3833,13 +4231,18 @@
           <t>Comprendre le circuit de l'argent.</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr"/>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Retenue sur salaire = le Trésor prélève la cotisation sur la solde et la reverse au FPPN. Note les autres modes cités.</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="B15" s="5" t="n">
@@ -3860,13 +4263,18 @@
           <t>Apprécier la régularité des ressources.</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr"/>
-      <c r="G15" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : chaque mois, avec un décalage. Alerte : retards de plusieurs mois.</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr"/>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="B16" s="5" t="n">
@@ -3889,15 +4297,20 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
+          <t>Attendu : un montant et une période. La presse a évoqué plus de 3 milliards FCFA. Demande l'état détaillé.</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
           <t>État des cotisations non reversées</t>
         </is>
       </c>
-      <c r="G16" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr"/>
+      <c r="H16" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="B17" s="14" t="inlineStr">
@@ -3910,7 +4323,8 @@
       <c r="E17" s="15" t="n"/>
       <c r="F17" s="15" t="n"/>
       <c r="G17" s="15" t="n"/>
-      <c r="H17" s="16" t="n"/>
+      <c r="H17" s="15" t="n"/>
+      <c r="I17" s="16" t="n"/>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="B18" s="5" t="n">
@@ -3931,15 +4345,20 @@
           <t>Données de base de tous mes calculs.</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr"/>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : des nombres précis par catégorie. Alerte : « environ », sans fichier à l'appui.</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19" ht="46" customHeight="1">
       <c r="B19" s="5" t="n">
         <v>9</v>
       </c>
@@ -3958,13 +4377,18 @@
           <t>Vérifier que les données nécessaires existent.</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr"/>
-      <c r="G19" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Statut = actif, retraité, sorti ou décédé. Attendu : oui. Si une donnée manque, demande où la trouver (fichier de la solde, ressources humaines).</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr"/>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="B20" s="5" t="n">
@@ -3985,13 +4409,18 @@
           <t>Apprécier la fiabilité des effectifs.</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr"/>
-      <c r="G20" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : mise à jour chaque mois avec la solde. Alerte : mise à jour rare, décédés encore présents.</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr"/>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="B21" s="5" t="n">
@@ -4012,15 +4441,20 @@
           <t>Contrôler l'exhaustivité des effectifs.</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr"/>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : oui, rapprochement avec la liste de la solde. Alerte : fichiers différents jamais rapprochés.</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr"/>
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr"/>
-    </row>
-    <row r="22" ht="32" customHeight="1">
+      <c r="I21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22" ht="46" customHeight="1">
       <c r="B22" s="5" t="n">
         <v>12</v>
       </c>
@@ -4041,15 +4475,20 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
+          <t>Attendu : oui, ou seulement le fichier actuel. Dans ce cas, demande les sorties datées pour reconstituer les années passées.</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
           <t>Fichiers des mutualistes 2019-2026 (Excel)</t>
         </is>
       </c>
-      <c r="G22" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr"/>
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr"/>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="B23" s="5" t="n">
@@ -4072,15 +4511,20 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
+          <t>Ayants droit = conjoint et enfants couverts. Attendu : oui avec dates de naissance, ou en partie.</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
           <t>Fichier des ayants droit</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr"/>
+      <c r="I23" s="6" t="inlineStr"/>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="B24" s="5" t="n">
@@ -4103,15 +4547,20 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
+          <t>Attendu : des chiffres par année. Ils servent à projeter l'effectif futur.</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
           <t>État des mouvements d'effectifs</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="B25" s="14" t="inlineStr">
@@ -4124,7 +4573,8 @@
       <c r="E25" s="15" t="n"/>
       <c r="F25" s="15" t="n"/>
       <c r="G25" s="15" t="n"/>
-      <c r="H25" s="16" t="n"/>
+      <c r="H25" s="15" t="n"/>
+      <c r="I25" s="16" t="n"/>
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="B26" s="5" t="n">
@@ -4145,15 +4595,20 @@
           <t>Savoir si l'épargne est liée aux cotisations.</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr"/>
-      <c r="G26" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr"/>
-    </row>
-    <row r="27" ht="32" customHeight="1">
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : oui (une part fixe va à l'épargne) ou non (épargne séparée).</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr"/>
+      <c r="H26" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27" ht="46" customHeight="1">
       <c r="B27" s="5" t="n">
         <v>16</v>
       </c>
@@ -4174,15 +4629,20 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
+          <t>Compte individuel = solde propre à chaque mutualiste. Attendu : oui, dans un logiciel. Alerte : seulement un total global.</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
           <t>Comptes individuels d'épargne</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr"/>
+      <c r="I27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="B28" s="14" t="inlineStr">
@@ -4195,7 +4655,8 @@
       <c r="E28" s="15" t="n"/>
       <c r="F28" s="15" t="n"/>
       <c r="G28" s="15" t="n"/>
-      <c r="H28" s="16" t="n"/>
+      <c r="H28" s="15" t="n"/>
+      <c r="I28" s="16" t="n"/>
     </row>
     <row r="29" ht="32" customHeight="1">
       <c r="B29" s="5" t="n">
@@ -4216,13 +4677,18 @@
           <t>Apprécier la fiabilité des cotisations enregistrées.</t>
         </is>
       </c>
-      <c r="F29" s="6" t="inlineStr"/>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : le comptable ou un chef de service, chaque mois. Alerte : aucun contrôle.</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr"/>
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H29" s="6" t="inlineStr"/>
+      <c r="I29" s="6" t="inlineStr"/>
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="B30" s="5" t="n">
@@ -4243,13 +4709,18 @@
           <t>Repérer des pertes de ressources.</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr"/>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : un tableau des écarts avec explication. Alerte : écarts non suivis.</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr"/>
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr"/>
+      <c r="I30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="B31" s="14" t="inlineStr">
@@ -4262,7 +4733,8 @@
       <c r="E31" s="15" t="n"/>
       <c r="F31" s="15" t="n"/>
       <c r="G31" s="15" t="n"/>
-      <c r="H31" s="16" t="n"/>
+      <c r="H31" s="15" t="n"/>
+      <c r="I31" s="16" t="n"/>
     </row>
     <row r="32" ht="32" customHeight="1">
       <c r="B32" s="5" t="n">
@@ -4283,15 +4755,20 @@
           <t>Organiser l'extraction des données.</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr"/>
-      <c r="G32" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr"/>
-    </row>
-    <row r="33" ht="32" customHeight="1">
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : nom du logiciel et du service. Note le nom du contact pour les extractions.</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr"/>
+      <c r="H32" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33" ht="46" customHeight="1">
       <c r="B33" s="5" t="n">
         <v>20</v>
       </c>
@@ -4312,15 +4789,20 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
+          <t>Attendu : un âge fixé par les textes de la police, parfois selon le grade. Demande la référence du texte.</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
           <t>Texte de référence</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr"/>
+      <c r="I33" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="B35" s="2" t="inlineStr">
@@ -4359,21 +4841,21 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B36:H36"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B39:H39"/>
-    <mergeCell ref="B31:H31"/>
-    <mergeCell ref="B38:H38"/>
-    <mergeCell ref="B25:H25"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B37:H37"/>
-    <mergeCell ref="B28:H28"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B39:I39"/>
+    <mergeCell ref="B25:I25"/>
+    <mergeCell ref="B38:I38"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="B37:I37"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B17:I17"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G8:G34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H8:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4389,17 +4871,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:H30"/>
+  <dimension ref="B2:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -4426,7 +4909,7 @@
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usage interne : la colonne « À quoi elle sert » est réservée à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
+          <t>Usage interne : les colonnes « À quoi elle sert » et « Explication » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
         </is>
       </c>
     </row>
@@ -4453,15 +4936,20 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
+          <t>Explication et réponses attendues (usage interne)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
           <t>Document à demander</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Réponse obtenue</t>
         </is>
@@ -4478,7 +4966,8 @@
       <c r="E8" s="15" t="n"/>
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
-      <c r="H8" s="16" t="n"/>
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="16" t="n"/>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="B9" s="5" t="n">
@@ -4499,13 +4988,18 @@
           <t>Organiser l'extraction des données.</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : nom du logiciel, fichiers Excel ou papier.</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="B10" s="5" t="n">
@@ -4528,17 +5022,22 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
+          <t>Extraction = export des données vers Excel. Attendu : oui, ou seulement la situation actuelle.</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
           <t>Extractions Excel</t>
         </is>
       </c>
-      <c r="G10" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="32" customHeight="1">
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="46" customHeight="1">
       <c r="B11" s="5" t="n">
         <v>3</v>
       </c>
@@ -4557,13 +5056,18 @@
           <t>Savoir si les situations passées peuvent être reconstituées.</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr"/>
-      <c r="G11" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Historique = données passées conservées. Écrasé = l'ancienne version disparaît. Si écrasé, les années passées sont à reconstituer.</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="B12" s="5" t="n">
@@ -4584,15 +5088,20 @@
           <t>Rapprocher mutualistes, prestations et épargne.</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Matricule = identifiant unique du policier. Alerte : nom seul, risque de doublons.</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13" ht="18" customHeight="1">
+      <c r="I12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="32" customHeight="1">
       <c r="B13" s="5" t="n">
         <v>5</v>
       </c>
@@ -4611,13 +5120,18 @@
           <t>Planifier la réception des données.</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr"/>
-      <c r="G13" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : un nom et un délai en jours.</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="14" t="inlineStr">
@@ -4630,9 +5144,10 @@
       <c r="E14" s="15" t="n"/>
       <c r="F14" s="15" t="n"/>
       <c r="G14" s="15" t="n"/>
-      <c r="H14" s="16" t="n"/>
-    </row>
-    <row r="15" ht="32" customHeight="1">
+      <c r="H14" s="15" t="n"/>
+      <c r="I14" s="16" t="n"/>
+    </row>
+    <row r="15" ht="46" customHeight="1">
       <c r="B15" s="5" t="n">
         <v>6</v>
       </c>
@@ -4651,15 +5166,20 @@
           <t>Planifier les calculs à cette date.</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr"/>
-      <c r="G15" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr"/>
-    </row>
-    <row r="16" ht="32" customHeight="1">
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Situation intermédiaire = comptes arrêtés au 31/08/2026. Attendu : une date (l'offre prévoit la semaine 3).</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16" ht="46" customHeight="1">
       <c r="B16" s="5" t="n">
         <v>7</v>
       </c>
@@ -4678,13 +5198,18 @@
           <t>Savoir quelles règles de provisionnement s'appliquent.</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr"/>
-      <c r="G16" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>PCMS = plan comptable des mutuelles sociales. SYSCOHADA = plan comptable général OHADA. Attendu : l'un ou l'autre, avec l'année d'un éventuel changement.</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr"/>
     </row>
     <row r="17" ht="32" customHeight="1">
       <c r="B17" s="5" t="n">
@@ -4705,13 +5230,18 @@
           <t>Recouper avec l'entretien provisionnements.</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr"/>
-      <c r="G17" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : la méthode, qui calcule, qui valide. À comparer avec l'entretien provisionnements.</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr"/>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="B18" s="5" t="n">
@@ -4732,13 +5262,18 @@
           <t>Mesurer l'effet sur les placements et la trésorerie.</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr"/>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : trésorerie, placements, emprunt ou apport de l'État. Note la source.</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr"/>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="B19" s="5" t="n">
@@ -4761,15 +5296,20 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
+          <t>Attendu : un budget annuel, plus rarement sur plusieurs années.</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
           <t>Budgets et prévisions</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr"/>
+      <c r="I19" s="6" t="inlineStr"/>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="B20" s="5" t="n">
@@ -4790,13 +5330,18 @@
           <t>Intégrer les frais dans les calculs.</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr"/>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Frais de gestion = coûts de fonctionnement. Attendu : souvent un total global, sans détail par activité.</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="B21" s="14" t="inlineStr">
@@ -4809,9 +5354,10 @@
       <c r="E21" s="15" t="n"/>
       <c r="F21" s="15" t="n"/>
       <c r="G21" s="15" t="n"/>
-      <c r="H21" s="16" t="n"/>
-    </row>
-    <row r="22" ht="32" customHeight="1">
+      <c r="H21" s="15" t="n"/>
+      <c r="I21" s="16" t="n"/>
+    </row>
+    <row r="22" ht="46" customHeight="1">
       <c r="B22" s="5" t="n">
         <v>12</v>
       </c>
@@ -4832,15 +5378,20 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
+          <t>Attendu : statuts datés et versions successives. Alerte : textes jugés caducs lors d'une AG extraordinaire.</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
           <t>Statuts et règlements successifs</t>
         </is>
       </c>
-      <c r="G22" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr"/>
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr"/>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="B23" s="5" t="n">
@@ -4863,15 +5414,20 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
+          <t>Litige = désaccord en réclamation ou en justice. Attendu : un nombre et des montants.</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
           <t>État des litiges</t>
         </is>
       </c>
-      <c r="G23" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr"/>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr"/>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="B24" s="5" t="n">
@@ -4894,15 +5450,20 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
+          <t>Agrément = autorisation de fonctionner délivrée par l'AIRMS. Attendu : oui, avec un numéro.</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
           <t>Agrément et courriers de l'AIRMS</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr"/>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="B25" s="5" t="n">
@@ -4925,15 +5486,20 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
+          <t>CGRAE = caisse de retraite des fonctionnaires. Attendu : une convention signée et datée.</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
           <t>Convention CGRAE</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr"/>
+      <c r="I25" s="6" t="inlineStr"/>
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="B26" s="5" t="n">
@@ -4954,13 +5520,18 @@
           <t>Apprécier les risques sur ces actifs.</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr"/>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : un texte qui autorise le crédit (statuts, agrément). Alerte : activité sans base claire.</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr"/>
+      <c r="I26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="B27" s="14" t="inlineStr">
@@ -4973,7 +5544,8 @@
       <c r="E27" s="15" t="n"/>
       <c r="F27" s="15" t="n"/>
       <c r="G27" s="15" t="n"/>
-      <c r="H27" s="16" t="n"/>
+      <c r="H27" s="15" t="n"/>
+      <c r="I27" s="16" t="n"/>
     </row>
     <row r="28" ht="32" customHeight="1">
       <c r="B28" s="5" t="n">
@@ -4996,15 +5568,20 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
+          <t>Inventaire = liste des biens avec leur valeur. Attendu : une liste, souvent sans valeur à jour.</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
           <t>Inventaire immobilier</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr"/>
+      <c r="I28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="B29" s="14" t="inlineStr">
@@ -5017,7 +5594,8 @@
       <c r="E29" s="15" t="n"/>
       <c r="F29" s="15" t="n"/>
       <c r="G29" s="15" t="n"/>
-      <c r="H29" s="16" t="n"/>
+      <c r="H29" s="15" t="n"/>
+      <c r="I29" s="16" t="n"/>
     </row>
     <row r="30" ht="46" customHeight="1">
       <c r="B30" s="5" t="n">
@@ -5040,28 +5618,33 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
+          <t>Attendu : des rapports avec constats. Note ceux qui touchent tes sujets.</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
           <t>Rapports d'audit interne</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr"/>
+      <c r="I30" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B27:H27"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B29:H29"/>
-    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B4:I4"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G8:G31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H8:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5077,18 +5660,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I26"/>
+  <dimension ref="B2:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -5115,7 +5699,7 @@
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usage interne : la colonne « À quoi elle sert » est réservée à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
+          <t>Usage interne : les colonnes « À quoi elle sert » et « Explication » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
         </is>
       </c>
     </row>
@@ -5142,20 +5726,25 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
+          <t>Explication et réponses attendues (usage interne)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
           <t>Document à demander</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Interlocuteur supposé</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -5173,7 +5762,8 @@
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
       <c r="H8" s="15" t="n"/>
-      <c r="I8" s="16" t="n"/>
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="16" t="n"/>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="B9" s="5" t="n">
@@ -5196,22 +5786,27 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
+          <t>Encours = capital restant dû. Attendu : une liste par emprunteur. Alerte : seulement un total.</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
           <t>Encours par emprunteur</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>Directeur du Grenier du Policier ; Caisse de crédit mutuel (rattachée au DGA)</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
+      <c r="J9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
       <c r="B10" s="5" t="n">
         <v>2</v>
       </c>
@@ -5232,20 +5827,25 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
+          <t>Impayé = échéance non remboursée. Ancienneté = depuis combien de temps. Attendu : remboursement par retenue sur solde, impayés classés par durée.</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
           <t>Échéancier et impayés</t>
         </is>
       </c>
-      <c r="G10" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Directeur du Grenier du Policier</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="B11" s="5" t="n">
@@ -5268,20 +5868,25 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
+          <t>Attendu : un taux annuel et une durée par type de prêt.</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
           <t>Conditions des prêts</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Directeur du Grenier du Policier</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="B12" s="14" t="inlineStr">
@@ -5295,9 +5900,10 @@
       <c r="F12" s="15" t="n"/>
       <c r="G12" s="15" t="n"/>
       <c r="H12" s="15" t="n"/>
-      <c r="I12" s="16" t="n"/>
-    </row>
-    <row r="13" ht="32" customHeight="1">
+      <c r="I12" s="15" t="n"/>
+      <c r="J12" s="16" t="n"/>
+    </row>
+    <row r="13" ht="46" customHeight="1">
       <c r="B13" s="5" t="n">
         <v>4</v>
       </c>
@@ -5318,22 +5924,27 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
+          <t>Allocation = somme versée lors d'un événement (décès, naissance, mariage). Attendu : une liste et des montants.</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
           <t>Barèmes des aides</t>
         </is>
       </c>
-      <c r="G13" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>Chef du service des affaires sociales</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14" ht="32" customHeight="1">
+      <c r="J13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14" ht="46" customHeight="1">
       <c r="B14" s="5" t="n">
         <v>5</v>
       </c>
@@ -5354,22 +5965,27 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
+          <t>Prise en charge = part des frais payée par le FPPN. Attendu : un taux, des plafonds, un réseau de soins.</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
           <t>Statistiques des soins</t>
         </is>
       </c>
-      <c r="G14" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>Chef du service médical</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr"/>
-    </row>
-    <row r="15" ht="32" customHeight="1">
+      <c r="J14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15" ht="46" customHeight="1">
       <c r="B15" s="5" t="n">
         <v>6</v>
       </c>
@@ -5390,20 +6006,25 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
+          <t>Attendu : facture interne ou budget global. Sert à isoler le coût réel des soins.</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
           <t>Comptes du centre médical</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>Responsable du CM-FPPN</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="B16" s="14" t="inlineStr">
@@ -5417,7 +6038,8 @@
       <c r="F16" s="15" t="n"/>
       <c r="G16" s="15" t="n"/>
       <c r="H16" s="15" t="n"/>
-      <c r="I16" s="16" t="n"/>
+      <c r="I16" s="15" t="n"/>
+      <c r="J16" s="16" t="n"/>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="B17" s="5" t="n">
@@ -5440,22 +6062,27 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
+          <t>Attendu : le nom du service et un fichier des soldes par mutualiste. Alerte : aucun suivi individuel.</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
           <t>Comptes individuels d'épargne</t>
         </is>
       </c>
-      <c r="G17" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>Gestionnaire de l'épargne (poste absent de l'organigramme ; probablement service comptabilité)</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
-    </row>
-    <row r="18" ht="32" customHeight="1">
+      <c r="J17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18" ht="46" customHeight="1">
       <c r="B18" s="5" t="n">
         <v>8</v>
       </c>
@@ -5476,20 +6103,25 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
+          <t>Attendu : nombre et montants par année. La presse cite 264 retraités et 410 millions FCFA en décembre 2025.</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
           <t>État des paiements d'épargne</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>Gestionnaire de l'épargne</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="B19" s="14" t="inlineStr">
@@ -5503,7 +6135,8 @@
       <c r="F19" s="15" t="n"/>
       <c r="G19" s="15" t="n"/>
       <c r="H19" s="15" t="n"/>
-      <c r="I19" s="16" t="n"/>
+      <c r="I19" s="15" t="n"/>
+      <c r="J19" s="16" t="n"/>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="B20" s="5" t="n">
@@ -5526,20 +6159,25 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
+          <t>Attendu : valeur d'achat ou d'expertise, loyers perçus. Alerte : biens jamais évalués.</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
           <t>Évaluations et revenus</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>Responsable patrimoine et projets immobiliers (rattaché au service juridique)</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="B21" s="14" t="inlineStr">
@@ -5553,7 +6191,8 @@
       <c r="F21" s="15" t="n"/>
       <c r="G21" s="15" t="n"/>
       <c r="H21" s="15" t="n"/>
-      <c r="I21" s="16" t="n"/>
+      <c r="I21" s="15" t="n"/>
+      <c r="J21" s="16" t="n"/>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="B22" s="5" t="n">
@@ -5576,20 +6215,25 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
+          <t>PV = procès-verbal, compte rendu officiel d'une réunion. Attendu : une liste des décisions avec leurs dates.</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
           <t>Procès-verbaux et décisions</t>
         </is>
       </c>
-      <c r="G22" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>Chef de cabinet ; secrétariat de direction</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr"/>
+      <c r="J22" s="6" t="inlineStr"/>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="B23" s="5" t="n">
@@ -5612,20 +6256,25 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
+          <t>Attendu : études internes ou de cabinets. Demande les copies.</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
           <t>Études existantes</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>Conseillers techniques du DG</t>
         </is>
       </c>
-      <c r="I23" s="6" t="inlineStr"/>
+      <c r="J23" s="6" t="inlineStr"/>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="B24" s="5" t="n">
@@ -5648,22 +6297,27 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
+          <t>Attendu : courriers, rapports de contrôle, injonctions.</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
           <t>Courriers de l'AIRMS</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
         <is>
           <t>Directeur général ; chef de cabinet</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25" ht="32" customHeight="1">
+      <c r="J24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25" ht="46" customHeight="1">
       <c r="B25" s="5" t="n">
         <v>13</v>
       </c>
@@ -5684,20 +6338,25 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
+          <t>Attendu : un âge fixé par les textes de la police, parfois selon le grade. Demande la référence du texte.</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
           <t>Texte de référence</t>
         </is>
       </c>
-      <c r="G25" s="17" t="inlineStr">
-        <is>
-          <t>Incontournable</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>Service du personnel du FPPN ; à défaut, DRH de la Police nationale</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="6" t="inlineStr"/>
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="B26" s="5" t="n">
@@ -5720,33 +6379,38 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
+          <t>Attendu : nombre de décès et d'invalidités par année. Souvent non disponible au FPPN.</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
           <t>Statistiques</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>Service des affaires sociales ; DRH de la Police nationale</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr"/>
+      <c r="J26" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B12:I12"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B16:I16"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B5:J5"/>
+    <mergeCell ref="B19:J19"/>
+    <mergeCell ref="B8:J8"/>
+    <mergeCell ref="B4:J4"/>
+    <mergeCell ref="B12:J12"/>
+    <mergeCell ref="B21:J21"/>
+    <mergeCell ref="B16:J16"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G8:G27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H8:H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Guides d'entretien FPPN : ajout des colonnes méthode, formule et source
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_Guides_entretiens_actuariat_20261016.xlsx
+++ b/FPPN_Guides_entretiens_actuariat_20261016.xlsx
@@ -1075,18 +1075,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I44"/>
+  <dimension ref="B2:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1113,7 +1116,7 @@
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usage interne : les colonnes « À quoi elle sert » et « Explication » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
+          <t>Usage interne : les colonnes marquées « interne » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
         </is>
       </c>
     </row>
@@ -1145,15 +1148,30 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
+          <t>Méthodes possibles (interne)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Formule (interne)</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Source et argument (interne)</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
           <t>Document à demander</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1171,7 +1189,10 @@
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
       <c r="H8" s="15" t="n"/>
-      <c r="I8" s="16" t="n"/>
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="16" t="n"/>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="B9" s="5" t="n">
@@ -1197,17 +1218,20 @@
           <t>Prestation = somme ou service versé par le FPPN. Attendu : allocation décès, aide invalidité, soins, épargne de fin de carrière, aides sociales. Note chaque prestation citée.</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>Liste des prestations et barèmes</t>
         </is>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="K9" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="B10" s="5" t="n">
@@ -1235,15 +1259,22 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
+          <t>Montant fixe, ou barème selon le grade ou l'ancienneté, avec ou sans plafond.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
           <t>Règlement des prestations</t>
         </is>
       </c>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="K10" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="B11" s="5" t="n">
@@ -1269,17 +1300,20 @@
           <t>Attendu : « non », ou des dates de changement avec une décision du conseil ou de l'AG. Alerte : changement sans décision écrite.</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>Décisions du conseil ou de l'AG</t>
         </is>
       </c>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="B12" s="5" t="n">
@@ -1305,15 +1339,30 @@
           <t>Capital = paiement unique. Rente = paiement régulier pendant plusieurs années. Si rente : demande la durée et les bénéficiaires.</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="17" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Capital : provision = montant dû. Rente : provision = valeur actuelle des paiements futurs.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>VA = Σ montant × p(t) ÷ (1+i)^t  (p(t) : probabilité de survie à t ; i : taux)</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>Code CIMA art. 334-2 et 338 : rentes calculées avec table de mortalité et taux ≤ 3,5 %. Référence technique.</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13" ht="46" customHeight="1">
+      <c r="L12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="60" customHeight="1">
       <c r="B13" s="5" t="n">
         <v>5</v>
       </c>
@@ -1337,15 +1386,30 @@
           <t>Attendu : oui pour la santé ou le décès, avec ou sans cotisation. Alerte : couverture à vie sans cotisation, donc engagement lourd non financé.</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr"/>
-      <c r="H13" s="17" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Promesse durable : valeur actuelle des coûts futurs par retraité.</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>VA = Σ montant × p(t) ÷ (1+i)^t  (p(t) : probabilité de survie à t ; i : taux)</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>Règlement d'exécution 004/2022/COM/UEMOA (1er juin 2022) : risques longs des mutuelles encadrés. Une promesse durable doit être évaluée.</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr"/>
+      <c r="K13" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14" ht="46" customHeight="1">
+      <c r="L13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14" ht="60" customHeight="1">
       <c r="B14" s="5" t="n">
         <v>6</v>
       </c>
@@ -1369,17 +1433,20 @@
           <t>CGRAE = caisse de retraite des fonctionnaires. Attendu : un partage des frais de soins des retraités entre la CGRAE et le FPPN. Demande la convention.</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>Convention avec la CGRAE</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="B15" s="5" t="n">
@@ -1406,12 +1473,15 @@
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr"/>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="B16" s="14" t="inlineStr">
@@ -1425,7 +1495,10 @@
       <c r="F16" s="15" t="n"/>
       <c r="G16" s="15" t="n"/>
       <c r="H16" s="15" t="n"/>
-      <c r="I16" s="16" t="n"/>
+      <c r="I16" s="15" t="n"/>
+      <c r="J16" s="15" t="n"/>
+      <c r="K16" s="15" t="n"/>
+      <c r="L16" s="16" t="n"/>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="B17" s="5" t="n">
@@ -1451,17 +1524,20 @@
           <t>Attendu : déclaration, dossier, vérification, validation, paiement. Repère les dates enregistrées à chaque étape.</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>Procédure de traitement</t>
         </is>
       </c>
-      <c r="H17" s="17" t="inlineStr">
+      <c r="K17" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr"/>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="B18" s="5" t="n">
@@ -1487,15 +1563,26 @@
           <t>Attendu : un délai en semaines ou en mois. Plus il est long, plus la provision pour dossiers en cours doit être élevée.</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr"/>
-      <c r="H18" s="17" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Délai moyen de règlement, calculé sur les dossiers payés.</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Délai moyen = moyenne (date de paiement − date de l'événement)</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr"/>
+      <c r="K18" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19" ht="46" customHeight="1">
+      <c r="L18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19" ht="60" customHeight="1">
       <c r="B19" s="5" t="n">
         <v>10</v>
       </c>
@@ -1519,13 +1606,28 @@
           <t>Tardif = événement survenu avant la clôture mais déclaré après. Attendu : un délai fixé par les règles, ou aucun. Alerte : déclarations plusieurs années après.</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr"/>
-      <c r="H19" s="17" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Tardifs estimés par la cadence de déclaration ou par Chain Ladder.</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Tardifs = charge totale estimée − dossiers connus</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Code CIMA art. 334-8 : la provision couvre les sinistres survenus et non payés, déclarés ou non. Référence technique.</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr"/>
+      <c r="K19" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr"/>
+      <c r="L19" s="6" t="inlineStr"/>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="B20" s="5" t="n">
@@ -1553,15 +1655,30 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
+          <t>Provision dossier par dossier (dossiers connus).</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Provision = Σ montants dus des dossiers non payés</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>Principe de prudence (SYSCOHADA révisé depuis 2018 ; PCMS) : toute dette connue à la clôture est enregistrée.</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
           <t>Liste des dossiers en attente</t>
         </is>
       </c>
-      <c r="H20" s="17" t="inlineStr">
+      <c r="K20" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr"/>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="B21" s="5" t="n">
@@ -1588,12 +1705,15 @@
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr"/>
-      <c r="H21" s="17" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr"/>
+      <c r="I21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="inlineStr"/>
+      <c r="K21" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I21" s="6" t="inlineStr"/>
+      <c r="L21" s="6" t="inlineStr"/>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="B22" s="5" t="n">
@@ -1621,15 +1741,30 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
+          <t>Comparer les arriérés payés aux dettes inscrites au bilan de l'année d'origine.</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Écart = montant payé − dette inscrite à l'origine</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>ISA 540 révisée (exercices ouverts dès le 15/12/2019) : comparer les estimations passées aux montants réels.</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
           <t>État des arriérés apurés</t>
         </is>
       </c>
-      <c r="H22" s="17" t="inlineStr">
+      <c r="K22" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="B23" s="14" t="inlineStr">
@@ -1643,9 +1778,12 @@
       <c r="F23" s="15" t="n"/>
       <c r="G23" s="15" t="n"/>
       <c r="H23" s="15" t="n"/>
-      <c r="I23" s="16" t="n"/>
-    </row>
-    <row r="24" ht="46" customHeight="1">
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="16" t="n"/>
+    </row>
+    <row r="24" ht="60" customHeight="1">
       <c r="B24" s="5" t="n">
         <v>14</v>
       </c>
@@ -1669,17 +1807,20 @@
           <t>Tiers payant = le FPPN paie directement la clinique. Remboursement = le mutualiste avance puis est remboursé. Attendu : l'un, l'autre ou les deux.</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr"/>
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>Conventions avec les prestataires</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr"/>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="B25" s="5" t="n">
@@ -1705,13 +1846,24 @@
           <t>Attendu : un délai en semaines ou en mois. Plus il est long, plus il reste de soins non facturés à la clôture.</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr"/>
-      <c r="H25" s="17" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Soins non facturés estimés avec le délai moyen de facturation.</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>Provision = coût mensuel moyen × délai moyen (en mois)</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="6" t="inlineStr"/>
+      <c r="K25" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr"/>
     </row>
     <row r="26" ht="46" customHeight="1">
       <c r="B26" s="5" t="n">
@@ -1738,12 +1890,15 @@
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr"/>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr"/>
+      <c r="I26" s="6" t="inlineStr"/>
+      <c r="J26" s="6" t="inlineStr"/>
+      <c r="K26" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="B27" s="14" t="inlineStr">
@@ -1757,7 +1912,10 @@
       <c r="F27" s="15" t="n"/>
       <c r="G27" s="15" t="n"/>
       <c r="H27" s="15" t="n"/>
-      <c r="I27" s="16" t="n"/>
+      <c r="I27" s="15" t="n"/>
+      <c r="J27" s="15" t="n"/>
+      <c r="K27" s="15" t="n"/>
+      <c r="L27" s="16" t="n"/>
     </row>
     <row r="28" ht="46" customHeight="1">
       <c r="B28" s="5" t="n">
@@ -1784,12 +1942,15 @@
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr"/>
-      <c r="H28" s="17" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr"/>
+      <c r="I28" s="6" t="inlineStr"/>
+      <c r="J28" s="6" t="inlineStr"/>
+      <c r="K28" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr"/>
     </row>
     <row r="29" ht="46" customHeight="1">
       <c r="B29" s="5" t="n">
@@ -1817,17 +1978,32 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
+          <t>Triangle de paiements : années de survenance × années de paiement.</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>C(i,j) = paiements cumulés de l'année i, j années après</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>Méthode Chain Ladder : pratique actuarielle courante pour estimer les tardifs.</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
           <t>Fichier des prestations payées (Excel)</t>
         </is>
       </c>
-      <c r="H29" s="17" t="inlineStr">
+      <c r="K29" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I29" s="6" t="inlineStr"/>
-    </row>
-    <row r="30" ht="32" customHeight="1">
+      <c r="L29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30" ht="46" customHeight="1">
       <c r="B30" s="5" t="n">
         <v>19</v>
       </c>
@@ -1852,14 +2028,17 @@
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr"/>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr"/>
+      <c r="I30" s="6" t="inlineStr"/>
+      <c r="J30" s="6" t="inlineStr"/>
+      <c r="K30" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31" ht="32" customHeight="1">
+      <c r="L30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31" ht="46" customHeight="1">
       <c r="B31" s="5" t="n">
         <v>20</v>
       </c>
@@ -1885,15 +2064,26 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
+          <t>Ratio prestations sur cotisations, par année.</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>S/C = prestations de l'année ÷ cotisations de l'année</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr"/>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
           <t>Tableaux de bord des prestations</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="K31" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr"/>
+      <c r="L31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="B32" s="14" t="inlineStr">
@@ -1907,7 +2097,10 @@
       <c r="F32" s="15" t="n"/>
       <c r="G32" s="15" t="n"/>
       <c r="H32" s="15" t="n"/>
-      <c r="I32" s="16" t="n"/>
+      <c r="I32" s="15" t="n"/>
+      <c r="J32" s="15" t="n"/>
+      <c r="K32" s="15" t="n"/>
+      <c r="L32" s="16" t="n"/>
     </row>
     <row r="33" ht="32" customHeight="1">
       <c r="B33" s="5" t="n">
@@ -1934,12 +2127,15 @@
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr"/>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr"/>
+      <c r="I33" s="6" t="inlineStr"/>
+      <c r="J33" s="6" t="inlineStr"/>
+      <c r="K33" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I33" s="6" t="inlineStr"/>
+      <c r="L33" s="6" t="inlineStr"/>
     </row>
     <row r="34" ht="46" customHeight="1">
       <c r="B34" s="5" t="n">
@@ -1966,12 +2162,15 @@
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr"/>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="H34" s="6" t="inlineStr"/>
+      <c r="I34" s="6" t="inlineStr"/>
+      <c r="J34" s="6" t="inlineStr"/>
+      <c r="K34" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr"/>
+      <c r="L34" s="6" t="inlineStr"/>
     </row>
     <row r="35" ht="32" customHeight="1">
       <c r="B35" s="5" t="n">
@@ -1998,12 +2197,15 @@
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr"/>
-      <c r="H35" s="6" t="inlineStr">
+      <c r="H35" s="6" t="inlineStr"/>
+      <c r="I35" s="6" t="inlineStr"/>
+      <c r="J35" s="6" t="inlineStr"/>
+      <c r="K35" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I35" s="6" t="inlineStr"/>
+      <c r="L35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="B36" s="14" t="inlineStr">
@@ -2017,7 +2219,10 @@
       <c r="F36" s="15" t="n"/>
       <c r="G36" s="15" t="n"/>
       <c r="H36" s="15" t="n"/>
-      <c r="I36" s="16" t="n"/>
+      <c r="I36" s="15" t="n"/>
+      <c r="J36" s="15" t="n"/>
+      <c r="K36" s="15" t="n"/>
+      <c r="L36" s="16" t="n"/>
     </row>
     <row r="37" ht="46" customHeight="1">
       <c r="B37" s="5" t="n">
@@ -2045,17 +2250,32 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
+          <t>Provision si la perte est probable et chiffrable.</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>Provision = meilleure estimation de la somme à payer</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>Principe de prudence (SYSCOHADA révisé depuis 2018 ; PCMS) : un risque probable donne lieu à provision.</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
           <t>État des litiges</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="K37" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I37" s="6" t="inlineStr"/>
-    </row>
-    <row r="38" ht="46" customHeight="1">
+      <c r="L37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38" ht="60" customHeight="1">
       <c r="B38" s="5" t="n">
         <v>25</v>
       </c>
@@ -2080,12 +2300,15 @@
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr"/>
-      <c r="H38" s="6" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr"/>
+      <c r="I38" s="6" t="inlineStr"/>
+      <c r="J38" s="6" t="inlineStr"/>
+      <c r="K38" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I38" s="6" t="inlineStr"/>
+      <c r="L38" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="B40" s="2" t="inlineStr">
@@ -2124,21 +2347,21 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B44:I44"/>
-    <mergeCell ref="B16:I16"/>
-    <mergeCell ref="B42:I42"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B36:I36"/>
-    <mergeCell ref="B41:I41"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B4:L4"/>
+    <mergeCell ref="B43:L43"/>
+    <mergeCell ref="B41:L41"/>
+    <mergeCell ref="B44:L44"/>
+    <mergeCell ref="B16:L16"/>
+    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="B42:L42"/>
+    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="B32:L32"/>
+    <mergeCell ref="B23:L23"/>
+    <mergeCell ref="B27:L27"/>
+    <mergeCell ref="B8:L8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H8:H39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K8:K39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2154,18 +2377,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I41"/>
+  <dimension ref="B2:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -2192,7 +2418,7 @@
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usage interne : les colonnes « À quoi elle sert » et « Explication » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
+          <t>Usage interne : les colonnes marquées « interne » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
         </is>
       </c>
     </row>
@@ -2224,15 +2450,30 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
+          <t>Méthodes possibles (interne)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Formule (interne)</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Source et argument (interne)</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
           <t>Document à demander</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2250,9 +2491,12 @@
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
       <c r="H8" s="15" t="n"/>
-      <c r="I8" s="16" t="n"/>
-    </row>
-    <row r="9" ht="46" customHeight="1">
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="16" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
       <c r="B9" s="5" t="n">
         <v>1</v>
       </c>
@@ -2278,17 +2522,28 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
+          <t>Prestations à payer, tardifs, épargne, cotisations non acquises, créances douteuses.</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Règlement 03/2012/CM/UEMOA (PCMS) : plan comptable propre aux mutuelles sociales.</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
           <t>Détail des provisions par nature</t>
         </is>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="K9" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="46" customHeight="1">
+      <c r="L9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
       <c r="B10" s="5" t="n">
         <v>2</v>
       </c>
@@ -2314,15 +2569,30 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
+          <t>Dossier par dossier, forfait, % des cotisations, Chain Ladder, valeur actuelle.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Chain Ladder : f(j) = Σ C(i,j+1) ÷ Σ C(i,j) ; charge totale = dernier cumul × produit des f</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>ISA 540 révisée (exercices ouverts dès le 15/12/2019) : méthode, hypothèses et données doivent être justifiées.</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
           <t>Note ou fichier de calcul</t>
         </is>
       </c>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="K10" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="B11" s="5" t="n">
@@ -2349,12 +2619,15 @@
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr"/>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="B12" s="5" t="n">
@@ -2380,13 +2653,24 @@
           <t>Attendu : non, ou un changement daté et expliqué. Alerte : changement sans explication.</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="17" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>La méthode reste la même chaque année, sauf changement justifié.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>Principe de permanence des méthodes (SYSCOHADA révisé ; PCMS).</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="B13" s="5" t="n">
@@ -2412,15 +2696,30 @@
           <t>Survenus non déclarés (IBNR) = événements arrivés avant la clôture, encore inconnus. Attendu : souvent « non ». Dans ce cas, les provisions sont probablement trop faibles.</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr"/>
-      <c r="H13" s="17" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Tardifs par Chain Ladder, ou par un ratio S/C si peu de données.</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Tardifs = charge totale − paiements cumulés − dossiers connus</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>Code CIMA art. 334-8 : sinistres survenus et non payés, déclarés ou non. Référence technique.</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr"/>
+      <c r="K13" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14" ht="46" customHeight="1">
+      <c r="L13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14" ht="60" customHeight="1">
       <c r="B14" s="5" t="n">
         <v>6</v>
       </c>
@@ -2444,13 +2743,28 @@
           <t>Engagement long = promesse sur plusieurs années, par exemple les soins des retraités à vie. Attendu : souvent « non ». Point important pour ton rapport.</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr"/>
-      <c r="H14" s="17" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Valeur actuelle des prestations futures promises aux retraités.</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>VA = Σ montant × p(t) ÷ (1+i)^t  (p(t) : probabilité de survie à t ; i : taux)</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>Règlement d'exécution 004/2022/COM/UEMOA (1er juin 2022) : risques longs des mutuelles encadrés. Code CIMA art. 334-2 en référence.</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr"/>
+      <c r="K14" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="B15" s="5" t="n">
@@ -2476,17 +2790,20 @@
           <t>Attendu : le plus souvent non, sinon le nom du cabinet et l'année. Demande le rapport.</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Rapport actuariel existant</t>
         </is>
       </c>
-      <c r="H15" s="17" t="inlineStr">
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr"/>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="B16" s="5" t="n">
@@ -2512,13 +2829,28 @@
           <t>Table de mortalité = probabilité de décès par âge (CIMA H par exemple). Taux d'actualisation = taux pour ramener un montant futur à aujourd'hui. Attendu : souvent aucune hypothèse.</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Table de mortalité, taux d'actualisation prudent, frais de gestion.</t>
+        </is>
+      </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
+          <t>Actualisation : VA = montant ÷ (1+i)^t</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>Code CIMA art. 338 (modifié en 2012) : tables CIMA H (décès) et CIMA F (vie), taux technique ≤ 3,5 %. Référence technique pour le FPPN.</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr"/>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr"/>
+      <c r="L16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="B17" s="14" t="inlineStr">
@@ -2532,7 +2864,10 @@
       <c r="F17" s="15" t="n"/>
       <c r="G17" s="15" t="n"/>
       <c r="H17" s="15" t="n"/>
-      <c r="I17" s="16" t="n"/>
+      <c r="I17" s="15" t="n"/>
+      <c r="J17" s="15" t="n"/>
+      <c r="K17" s="15" t="n"/>
+      <c r="L17" s="16" t="n"/>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="B18" s="5" t="n">
@@ -2558,15 +2893,30 @@
           <t>Boni = provision supérieure aux paiements réels. Mali = provision inférieure. Attendu : souvent pas de suivi. S'il existe, demande le tableau.</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr"/>
-      <c r="H18" s="17" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Test de liquidation : provision d'ouverture comparée aux paiements réels.</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Boni (+) ou mali (−) = provision début − (paiements de l'année + provision restante)</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>ISA 540 révisée (exercices ouverts dès le 15/12/2019) : revue des estimations de l'année précédente.</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr"/>
+      <c r="K18" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
+      <c r="L18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19" ht="46" customHeight="1">
       <c r="B19" s="5" t="n">
         <v>10</v>
       </c>
@@ -2591,14 +2941,17 @@
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr"/>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr"/>
+      <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="6" t="inlineStr"/>
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20" ht="46" customHeight="1">
+      <c r="L19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20" ht="60" customHeight="1">
       <c r="B20" s="5" t="n">
         <v>11</v>
       </c>
@@ -2622,13 +2975,24 @@
           <t>Référentiel = ensemble des règles comptables. Attendu : PCMS (plan comptable des mutuelles sociales) ou SYSCOHADA. Note l'année d'un éventuel changement.</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr"/>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>PCMS pour les mutuelles sociales ; SYSCOHADA pour ce que le PCMS ne traite pas.</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>Règlement 03/2012/CM/UEMOA (PCMS), exercices ouverts dès le 1er janvier 2014 (date à confirmer sur le texte).</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr"/>
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr"/>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="B21" s="5" t="n">
@@ -2656,17 +3020,32 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
+          <t>Comparer réserves et provisions aux ratios de l'AIRMS.</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Couverture = actifs admissibles ÷ engagements</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>Règlement 07/2009/CM/UEMOA (depuis le 1er juillet 2011) et Décision UEMOA n°05/2022 : ratios prudentiels.</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
           <t>Courriers de l'AIRMS</t>
         </is>
       </c>
-      <c r="H21" s="17" t="inlineStr">
+      <c r="K21" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I21" s="6" t="inlineStr"/>
-    </row>
-    <row r="22" ht="32" customHeight="1">
+      <c r="L21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22" ht="46" customHeight="1">
       <c r="B22" s="5" t="n">
         <v>13</v>
       </c>
@@ -2690,17 +3069,24 @@
           <t>Attendu : non, ou des courriers, mises en demeure, plan de redressement. Demande les courriers.</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr"/>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>L'AIRMS agrée, contrôle et peut sanctionner les mutuelles, jusqu'au retrait d'agrément.</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>Rapports de contrôle de l'AIRMS</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="K22" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="B23" s="14" t="inlineStr">
@@ -2714,7 +3100,10 @@
       <c r="F23" s="15" t="n"/>
       <c r="G23" s="15" t="n"/>
       <c r="H23" s="15" t="n"/>
-      <c r="I23" s="16" t="n"/>
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="16" t="n"/>
     </row>
     <row r="24" ht="46" customHeight="1">
       <c r="B24" s="5" t="n">
@@ -2740,17 +3129,20 @@
           <t>Attendu : épargne de fin de carrière, Plan Épargne Plus, ou aucun. Si aucun, les questions sur l'épargne tombent.</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr"/>
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>Description des produits d'épargne</t>
         </is>
       </c>
-      <c r="H24" s="17" t="inlineStr">
+      <c r="K24" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr"/>
     </row>
     <row r="25" ht="60" customHeight="1">
       <c r="B25" s="5" t="n">
@@ -2778,17 +3170,32 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
+          <t>Taux garanti : intérêts promis inclus dans la provision. Taux annuel : intérêts ajoutés une fois décidés.</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>Intérêts = solde × taux servi</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>Code CIMA art. 338 : taux garanti ≤ 3,5 % chez les assureurs. Repère de prudence.</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
           <t>Décisions fixant le taux</t>
         </is>
       </c>
-      <c r="H25" s="17" t="inlineStr">
+      <c r="K25" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26" ht="46" customHeight="1">
+      <c r="L25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26" ht="60" customHeight="1">
       <c r="B26" s="5" t="n">
         <v>16</v>
       </c>
@@ -2814,15 +3221,26 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
+          <t>Somme des comptes individuels = dette d'épargne au bilan.</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Solde fin = solde début + versements + intérêts − retraits</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr"/>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
           <t>Rapprochement comptes individuels et bilan</t>
         </is>
       </c>
-      <c r="H26" s="17" t="inlineStr">
+      <c r="K26" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="B27" s="14" t="inlineStr">
@@ -2836,7 +3254,10 @@
       <c r="F27" s="15" t="n"/>
       <c r="G27" s="15" t="n"/>
       <c r="H27" s="15" t="n"/>
-      <c r="I27" s="16" t="n"/>
+      <c r="I27" s="15" t="n"/>
+      <c r="J27" s="15" t="n"/>
+      <c r="K27" s="15" t="n"/>
+      <c r="L27" s="16" t="n"/>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="B28" s="5" t="n">
@@ -2862,13 +3283,24 @@
           <t>Situation au 31/08/2026 = comptes arrêtés en cours d'année, ce n'est pas une clôture annuelle. Attendu : une date. Alerte : provisions non recalculées à cette date.</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr"/>
-      <c r="H28" s="17" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Provisions recalculées à la date d'arrêté, comme en fin d'année.</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr"/>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>Offre technique : situation au 31/08/2026 à produire par le FPPN, prérequis du calendrier.</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr"/>
+      <c r="K28" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr"/>
     </row>
     <row r="29" ht="32" customHeight="1">
       <c r="B29" s="5" t="n">
@@ -2894,17 +3326,20 @@
           <t>Attendu : des fichiers Excel par année. Alerte : calculs non conservés.</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr"/>
+      <c r="H29" s="6" t="inlineStr"/>
+      <c r="I29" s="6" t="inlineStr"/>
+      <c r="J29" s="6" t="inlineStr">
         <is>
           <t>Fichiers de calcul 2019 à 2026</t>
         </is>
       </c>
-      <c r="H29" s="17" t="inlineStr">
+      <c r="K29" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I29" s="6" t="inlineStr"/>
+      <c r="L29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="B30" s="14" t="inlineStr">
@@ -2918,7 +3353,10 @@
       <c r="F30" s="15" t="n"/>
       <c r="G30" s="15" t="n"/>
       <c r="H30" s="15" t="n"/>
-      <c r="I30" s="16" t="n"/>
+      <c r="I30" s="15" t="n"/>
+      <c r="J30" s="15" t="n"/>
+      <c r="K30" s="15" t="n"/>
+      <c r="L30" s="16" t="n"/>
     </row>
     <row r="31" ht="32" customHeight="1">
       <c r="B31" s="5" t="n">
@@ -2945,12 +3383,15 @@
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr"/>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr"/>
+      <c r="I31" s="6" t="inlineStr"/>
+      <c r="J31" s="6" t="inlineStr"/>
+      <c r="K31" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr"/>
+      <c r="L31" s="6" t="inlineStr"/>
     </row>
     <row r="32" ht="32" customHeight="1">
       <c r="B32" s="5" t="n">
@@ -2977,12 +3418,15 @@
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr"/>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr"/>
+      <c r="I32" s="6" t="inlineStr"/>
+      <c r="J32" s="6" t="inlineStr"/>
+      <c r="K32" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I32" s="6" t="inlineStr"/>
+      <c r="L32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="B33" s="14" t="inlineStr">
@@ -2996,7 +3440,10 @@
       <c r="F33" s="15" t="n"/>
       <c r="G33" s="15" t="n"/>
       <c r="H33" s="15" t="n"/>
-      <c r="I33" s="16" t="n"/>
+      <c r="I33" s="15" t="n"/>
+      <c r="J33" s="15" t="n"/>
+      <c r="K33" s="15" t="n"/>
+      <c r="L33" s="16" t="n"/>
     </row>
     <row r="34" ht="46" customHeight="1">
       <c r="B34" s="5" t="n">
@@ -3022,13 +3469,24 @@
           <t>Attendu : non, la cotisation est globale ; ou une clé de répartition par garantie. Si non, la répartition devra être estimée.</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr"/>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>Sans clé : part estimée selon le coût de chaque garantie.</t>
+        </is>
+      </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
+          <t>Part de la garantie = coût de la garantie ÷ coût total</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr"/>
+      <c r="J34" s="6" t="inlineStr"/>
+      <c r="K34" s="6" t="inlineStr">
+        <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr"/>
+      <c r="L34" s="6" t="inlineStr"/>
     </row>
     <row r="35" ht="32" customHeight="1">
       <c r="B35" s="5" t="n">
@@ -3054,13 +3512,24 @@
           <t>Attendu : le plus souvent non. Si oui, note lesquels : ils servent directement à l'adossement.</t>
         </is>
       </c>
-      <c r="G35" s="6" t="inlineStr"/>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>Actifs mis en face des provisions, par échéance.</t>
+        </is>
+      </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
+          <t>Couverture = actifs affectés ÷ provisions</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr"/>
+      <c r="J35" s="6" t="inlineStr"/>
+      <c r="K35" s="6" t="inlineStr">
+        <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I35" s="6" t="inlineStr"/>
+      <c r="L35" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="B37" s="2" t="inlineStr">
@@ -3099,21 +3568,21 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B40:I40"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B39:I39"/>
-    <mergeCell ref="B38:I38"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B41:I41"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="B4:L4"/>
+    <mergeCell ref="B41:L41"/>
+    <mergeCell ref="B30:L30"/>
+    <mergeCell ref="B38:L38"/>
+    <mergeCell ref="B33:L33"/>
+    <mergeCell ref="B39:L39"/>
+    <mergeCell ref="B23:L23"/>
+    <mergeCell ref="B40:L40"/>
+    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="B27:L27"/>
+    <mergeCell ref="B8:L8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H8:H36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K8:K36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3129,18 +3598,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I37"/>
+  <dimension ref="B2:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -3167,7 +3639,7 @@
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usage interne : les colonnes « À quoi elle sert » et « Explication » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
+          <t>Usage interne : les colonnes marquées « interne » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
         </is>
       </c>
     </row>
@@ -3199,15 +3671,30 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
+          <t>Méthodes possibles (interne)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Formule (interne)</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Source et argument (interne)</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
           <t>Document à demander</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3225,7 +3712,10 @@
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
       <c r="H8" s="15" t="n"/>
-      <c r="I8" s="16" t="n"/>
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="16" t="n"/>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="B9" s="5" t="n">
@@ -3251,17 +3741,20 @@
           <t>Dépôt à terme = argent bloqué en banque pour une durée fixe. Obligation = prêt à un État ou une entreprise. Attendu : surtout des dépôts à terme et des comptes bancaires.</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>Inventaire des placements</t>
         </is>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="K9" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="B10" s="5" t="n">
@@ -3287,13 +3780,28 @@
           <t>Émetteur = celui qui émet le titre (État, entreprise). Alerte : une grande partie des placements dans une seule banque.</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr"/>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Mesurer la concentration par banque et par émetteur.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Part = placement dans l'établissement ÷ total des placements</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Code CIMA art. 335-4 : limites de concentration par émetteur. Référence technique.</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="B11" s="5" t="n">
@@ -3321,17 +3829,28 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
+          <t>Classer actifs et engagements par tranche : moins d'1 an, 1 à 5 ans, plus de 5 ans.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Écart = encaissements de la tranche − paiements de la tranche</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
           <t>Échéancier des placements</t>
         </is>
       </c>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12" ht="32" customHeight="1">
+      <c r="L11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12" ht="46" customHeight="1">
       <c r="B12" s="5" t="n">
         <v>4</v>
       </c>
@@ -3355,13 +3874,24 @@
           <t>Attendu : oui avec perte d'intérêts, ou non. Alerte : fonds bloqués alors que des paiements sont en retard.</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="17" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Actif liquide = disponible vite et sans perte importante.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Liquidité = actifs liquides ÷ paiements dus à moins d'1 an</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="B13" s="5" t="n">
@@ -3387,13 +3917,24 @@
           <t>Rendement = intérêts reçus ÷ montant placé. Attendu : un taux par année. Compare-le au taux servi sur l'épargne.</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Rendement annuel, comparé au taux servi aux épargnants.</t>
+        </is>
+      </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
+          <t>Rendement = revenus de l'année ÷ montant moyen placé</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr"/>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="14" t="inlineStr">
@@ -3407,9 +3948,12 @@
       <c r="F14" s="15" t="n"/>
       <c r="G14" s="15" t="n"/>
       <c r="H14" s="15" t="n"/>
-      <c r="I14" s="16" t="n"/>
-    </row>
-    <row r="15" ht="32" customHeight="1">
+      <c r="I14" s="15" t="n"/>
+      <c r="J14" s="15" t="n"/>
+      <c r="K14" s="15" t="n"/>
+      <c r="L14" s="16" t="n"/>
+    </row>
+    <row r="15" ht="46" customHeight="1">
       <c r="B15" s="5" t="n">
         <v>6</v>
       </c>
@@ -3433,19 +3977,26 @@
           <t>Attendu : un document validé par le conseil, ou des décisions au cas par cas du DG. Alerte : aucune règle.</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Règlement 07/2009/CM/UEMOA : gestion des ressources encadrée par des règles prudentielles.</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Politique de placement</t>
         </is>
       </c>
-      <c r="H15" s="17" t="inlineStr">
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr"/>
-    </row>
-    <row r="16" ht="46" customHeight="1">
+      <c r="L15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
       <c r="B16" s="5" t="n">
         <v>7</v>
       </c>
@@ -3469,13 +4020,28 @@
           <t>Adossement = faire correspondre les dates d'échéance des placements aux dates de paiement. Attendu : souvent « non ». Dans ce cas : risque de manque de liquidités.</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr"/>
-      <c r="H16" s="17" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Comparer les échéances des placements aux dates de paiement prévues.</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Durée moyenne = Σ (t × flux actualisé) ÷ Σ flux actualisés</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>Code CIMA art. 335 : engagements couverts à tout moment par des actifs équivalents. Référence technique.</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr"/>
+      <c r="K16" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr"/>
+      <c r="L16" s="6" t="inlineStr"/>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="B17" s="5" t="n">
@@ -3502,12 +4068,19 @@
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr"/>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>RE 004/2022/COM/UEMOA et Décision n°05/2022 : règles et ratios prudentiels des mutuelles.</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="B18" s="14" t="inlineStr">
@@ -3521,9 +4094,12 @@
       <c r="F18" s="15" t="n"/>
       <c r="G18" s="15" t="n"/>
       <c r="H18" s="15" t="n"/>
-      <c r="I18" s="16" t="n"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
+      <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="n"/>
+      <c r="K18" s="15" t="n"/>
+      <c r="L18" s="16" t="n"/>
+    </row>
+    <row r="19" ht="46" customHeight="1">
       <c r="B19" s="5" t="n">
         <v>9</v>
       </c>
@@ -3549,17 +4125,28 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
+          <t>Plan de trésorerie : encaissements et décaissements prévus, mois par mois.</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Trésorerie fin = trésorerie début + encaissements − décaissements</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
           <t>Prévisions de trésorerie</t>
         </is>
       </c>
-      <c r="H19" s="17" t="inlineStr">
+      <c r="K19" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20" ht="32" customHeight="1">
+      <c r="L19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20" ht="46" customHeight="1">
       <c r="B20" s="5" t="n">
         <v>10</v>
       </c>
@@ -3584,12 +4171,15 @@
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr"/>
-      <c r="H20" s="17" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr"/>
+      <c r="K20" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="B21" s="14" t="inlineStr">
@@ -3603,7 +4193,10 @@
       <c r="F21" s="15" t="n"/>
       <c r="G21" s="15" t="n"/>
       <c r="H21" s="15" t="n"/>
-      <c r="I21" s="16" t="n"/>
+      <c r="I21" s="15" t="n"/>
+      <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
+      <c r="L21" s="16" t="n"/>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="B22" s="5" t="n">
@@ -3631,15 +4224,30 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
+          <t>Créance non encaissée : exclue de la couverture ou dépréciée.</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Montant retenu = créance − dépréciation</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>Principe de prudence (SYSCOHADA révisé depuis 2018 ; PCMS) : une créance douteuse est dépréciée.</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
           <t>État des cotisations non reversées</t>
         </is>
       </c>
-      <c r="H22" s="17" t="inlineStr">
+      <c r="K22" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr"/>
     </row>
     <row r="23" ht="46" customHeight="1">
       <c r="B23" s="5" t="n">
@@ -3667,15 +4275,30 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
+          <t>Dépréciation des prêts selon l'ancienneté des impayés.</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>Taux d'impayés = impayés ÷ encours</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>Principe de prudence (SYSCOHADA révisé depuis 2018 ; PCMS) : un prêt douteux est déprécié.</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
           <t>Encours et impayés des prêts</t>
         </is>
       </c>
-      <c r="H23" s="17" t="inlineStr">
+      <c r="K23" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I23" s="6" t="inlineStr"/>
+      <c r="L23" s="6" t="inlineStr"/>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="B24" s="5" t="n">
@@ -3703,15 +4326,26 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
+          <t>Valeur d'expertise récente plutôt qu'un coût d'achat ancien.</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>Code CIMA art. 335-12 : principes d'évaluation des placements. Référence technique.</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
           <t>Dernière évaluation immobilière</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr"/>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="B25" s="5" t="n">
@@ -3738,12 +4372,15 @@
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr"/>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr"/>
+      <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="6" t="inlineStr"/>
+      <c r="K25" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="B26" s="14" t="inlineStr">
@@ -3757,7 +4394,10 @@
       <c r="F26" s="15" t="n"/>
       <c r="G26" s="15" t="n"/>
       <c r="H26" s="15" t="n"/>
-      <c r="I26" s="16" t="n"/>
+      <c r="I26" s="15" t="n"/>
+      <c r="J26" s="15" t="n"/>
+      <c r="K26" s="15" t="n"/>
+      <c r="L26" s="16" t="n"/>
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="B27" s="5" t="n">
@@ -3784,12 +4424,15 @@
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr"/>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr"/>
+      <c r="I27" s="6" t="inlineStr"/>
+      <c r="J27" s="6" t="inlineStr"/>
+      <c r="K27" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr"/>
+      <c r="L27" s="6" t="inlineStr"/>
     </row>
     <row r="28" ht="46" customHeight="1">
       <c r="B28" s="5" t="n">
@@ -3816,12 +4459,15 @@
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr"/>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr"/>
+      <c r="I28" s="6" t="inlineStr"/>
+      <c r="J28" s="6" t="inlineStr"/>
+      <c r="K28" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="B29" s="14" t="inlineStr">
@@ -3835,9 +4481,12 @@
       <c r="F29" s="15" t="n"/>
       <c r="G29" s="15" t="n"/>
       <c r="H29" s="15" t="n"/>
-      <c r="I29" s="16" t="n"/>
-    </row>
-    <row r="30" ht="32" customHeight="1">
+      <c r="I29" s="15" t="n"/>
+      <c r="J29" s="15" t="n"/>
+      <c r="K29" s="15" t="n"/>
+      <c r="L29" s="16" t="n"/>
+    </row>
+    <row r="30" ht="46" customHeight="1">
       <c r="B30" s="5" t="n">
         <v>17</v>
       </c>
@@ -3861,13 +4510,24 @@
           <t>Attendu : trésorerie, retrait de placements, emprunt ou apport de l'État. Note la source et le montant.</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr"/>
-      <c r="H30" s="17" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Comparer les placements avant et après l'apurement.</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>Variation = placements après − placements avant</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr"/>
+      <c r="J30" s="6" t="inlineStr"/>
+      <c r="K30" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr"/>
+      <c r="L30" s="6" t="inlineStr"/>
     </row>
     <row r="31" ht="46" customHeight="1">
       <c r="B31" s="5" t="n">
@@ -3893,13 +4553,24 @@
           <t>Nanti = bloqué en garantie d'un prêt. Attendu : non. Si oui, ces placements ne peuvent pas servir à payer les mutualistes.</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr"/>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>Exclure les actifs bloqués de la couverture.</t>
+        </is>
+      </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
+          <t>Actifs admissibles = total − actifs nantis</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr"/>
+      <c r="J31" s="6" t="inlineStr"/>
+      <c r="K31" s="6" t="inlineStr">
+        <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr"/>
+      <c r="L31" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="B33" s="2" t="inlineStr">
@@ -3938,21 +4609,21 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B18:I18"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B34:I34"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="B36:I36"/>
-    <mergeCell ref="B37:I37"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B26:I26"/>
+    <mergeCell ref="B35:L35"/>
+    <mergeCell ref="B4:L4"/>
+    <mergeCell ref="B26:L26"/>
+    <mergeCell ref="B21:L21"/>
+    <mergeCell ref="B29:L29"/>
+    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="B34:L34"/>
+    <mergeCell ref="B37:L37"/>
+    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="B14:L14"/>
+    <mergeCell ref="B18:L18"/>
+    <mergeCell ref="B8:L8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H8:H32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K8:K32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3968,18 +4639,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I39"/>
+  <dimension ref="B2:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -4006,7 +4680,7 @@
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usage interne : les colonnes « À quoi elle sert » et « Explication » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
+          <t>Usage interne : les colonnes marquées « interne » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
         </is>
       </c>
     </row>
@@ -4038,15 +4712,30 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
+          <t>Méthodes possibles (interne)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Formule (interne)</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Source et argument (interne)</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
           <t>Document à demander</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -4064,9 +4753,12 @@
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
       <c r="H8" s="15" t="n"/>
-      <c r="I8" s="16" t="n"/>
-    </row>
-    <row r="9" ht="46" customHeight="1">
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="16" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
       <c r="B9" s="5" t="n">
         <v>1</v>
       </c>
@@ -4090,17 +4782,20 @@
           <t>Catégories = actifs, retraités, autres membres. Attendu : montant fixe par mois ou pourcentage du salaire. Note les changements depuis 2020 et leur date.</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>Barème des cotisations 2020-2026</t>
         </is>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="K9" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="B10" s="5" t="n">
@@ -4126,13 +4821,24 @@
           <t>Clé de répartition = part de la cotisation affectée à chaque garantie. Attendu : souvent aucune. Dans ce cas, je l'estimerai.</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr"/>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Sans clé : part estimée selon le coût de chaque garantie.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Part = coût de la garantie ÷ coût total</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="B11" s="5" t="n">
@@ -4158,15 +4864,26 @@
           <t>Attendu : oui, prélevés sur la pension ou en paiement direct, ou non. Alerte : retraités couverts sans cotiser.</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr"/>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Comparer cotisations et coûts des retraités.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>S/C retraités = prestations des retraités ÷ cotisations des retraités</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12" ht="32" customHeight="1">
+      <c r="L11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12" ht="46" customHeight="1">
       <c r="B12" s="5" t="n">
         <v>4</v>
       </c>
@@ -4191,12 +4908,15 @@
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="14" t="inlineStr">
@@ -4210,7 +4930,10 @@
       <c r="F13" s="15" t="n"/>
       <c r="G13" s="15" t="n"/>
       <c r="H13" s="15" t="n"/>
-      <c r="I13" s="16" t="n"/>
+      <c r="I13" s="15" t="n"/>
+      <c r="J13" s="15" t="n"/>
+      <c r="K13" s="15" t="n"/>
+      <c r="L13" s="16" t="n"/>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="B14" s="5" t="n">
@@ -4237,12 +4960,15 @@
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr"/>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr"/>
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="B15" s="5" t="n">
@@ -4268,15 +4994,26 @@
           <t>Attendu : chaque mois, avec un décalage. Alerte : retards de plusieurs mois.</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr"/>
-      <c r="H15" s="17" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Mesurer le délai de reversement.</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Délai = date d'encaissement − mois de la retenue</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr"/>
-    </row>
-    <row r="16" ht="32" customHeight="1">
+      <c r="L15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16" ht="46" customHeight="1">
       <c r="B16" s="5" t="n">
         <v>7</v>
       </c>
@@ -4302,15 +5039,26 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
+          <t>Créance sur l'État : dépréciée ou exclue de la couverture tant qu'elle n'est pas encaissée.</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>Principe de prudence (SYSCOHADA révisé depuis 2018 ; PCMS) : une créance incertaine est dépréciée.</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
           <t>État des cotisations non reversées</t>
         </is>
       </c>
-      <c r="H16" s="17" t="inlineStr">
+      <c r="K16" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr"/>
+      <c r="L16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="B17" s="14" t="inlineStr">
@@ -4324,7 +5072,10 @@
       <c r="F17" s="15" t="n"/>
       <c r="G17" s="15" t="n"/>
       <c r="H17" s="15" t="n"/>
-      <c r="I17" s="16" t="n"/>
+      <c r="I17" s="15" t="n"/>
+      <c r="J17" s="15" t="n"/>
+      <c r="K17" s="15" t="n"/>
+      <c r="L17" s="16" t="n"/>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="B18" s="5" t="n">
@@ -4351,14 +5102,17 @@
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr"/>
-      <c r="H18" s="17" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr"/>
+      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr"/>
+      <c r="K18" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19" ht="46" customHeight="1">
+      <c r="L18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19" ht="60" customHeight="1">
       <c r="B19" s="5" t="n">
         <v>9</v>
       </c>
@@ -4382,15 +5136,30 @@
           <t>Statut = actif, retraité, sorti ou décédé. Attendu : oui. Si une donnée manque, demande où la trouver (fichier de la solde, ressources humaines).</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr"/>
-      <c r="H19" s="17" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Contrôles : âges plausibles, dates cohérentes, doublons.</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Âge = (date de clôture − date de naissance) ÷ 365,25</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>ISA 500 : les données utilisées doivent être fiables et complètes.</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr"/>
+      <c r="K19" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20" ht="32" customHeight="1">
+      <c r="L19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20" ht="46" customHeight="1">
       <c r="B20" s="5" t="n">
         <v>10</v>
       </c>
@@ -4415,14 +5184,17 @@
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr"/>
-      <c r="H20" s="17" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr"/>
+      <c r="K20" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21" ht="32" customHeight="1">
+      <c r="L20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21" ht="46" customHeight="1">
       <c r="B21" s="5" t="n">
         <v>11</v>
       </c>
@@ -4446,13 +5218,24 @@
           <t>Attendu : oui, rapprochement avec la liste de la solde. Alerte : fichiers différents jamais rapprochés.</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Rapprocher le fichier des mutualistes et la liste de la solde.</t>
+        </is>
+      </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
+          <t>Cotisations attendues = nombre de cotisants × cotisation</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="inlineStr"/>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I21" s="6" t="inlineStr"/>
+      <c r="L21" s="6" t="inlineStr"/>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="B22" s="5" t="n">
@@ -4480,17 +5263,28 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
+          <t>Reconstituer les effectifs passés avec les entrées et sorties datées.</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Effectif fin = effectif début + entrées − sorties</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr"/>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
           <t>Fichiers des mutualistes 2019-2026 (Excel)</t>
         </is>
       </c>
-      <c r="H22" s="17" t="inlineStr">
+      <c r="K22" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="32" customHeight="1">
+      <c r="L22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="46" customHeight="1">
       <c r="B23" s="5" t="n">
         <v>13</v>
       </c>
@@ -4514,17 +5308,20 @@
           <t>Ayants droit = conjoint et enfants couverts. Attendu : oui avec dates de naissance, ou en partie.</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr"/>
+      <c r="H23" s="6" t="inlineStr"/>
+      <c r="I23" s="6" t="inlineStr"/>
+      <c r="J23" s="6" t="inlineStr">
         <is>
           <t>Fichier des ayants droit</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="K23" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I23" s="6" t="inlineStr"/>
+      <c r="L23" s="6" t="inlineStr"/>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="B24" s="5" t="n">
@@ -4552,15 +5349,26 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
+          <t>Taux d'entrée et de sortie, base de la projection.</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Taux de sortie = sorties de l'année ÷ effectif de début</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr"/>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
           <t>État des mouvements d'effectifs</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="B25" s="14" t="inlineStr">
@@ -4574,7 +5382,10 @@
       <c r="F25" s="15" t="n"/>
       <c r="G25" s="15" t="n"/>
       <c r="H25" s="15" t="n"/>
-      <c r="I25" s="16" t="n"/>
+      <c r="I25" s="15" t="n"/>
+      <c r="J25" s="15" t="n"/>
+      <c r="K25" s="15" t="n"/>
+      <c r="L25" s="16" t="n"/>
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="B26" s="5" t="n">
@@ -4601,12 +5412,15 @@
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr"/>
-      <c r="H26" s="17" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr"/>
+      <c r="I26" s="6" t="inlineStr"/>
+      <c r="J26" s="6" t="inlineStr"/>
+      <c r="K26" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr"/>
     </row>
     <row r="27" ht="46" customHeight="1">
       <c r="B27" s="5" t="n">
@@ -4634,15 +5448,26 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
+          <t>Contrôle des comptes individuels.</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Solde fin = solde début + versements + intérêts − retraits</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr"/>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
           <t>Comptes individuels d'épargne</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="K27" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr"/>
+      <c r="L27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="B28" s="14" t="inlineStr">
@@ -4656,7 +5481,10 @@
       <c r="F28" s="15" t="n"/>
       <c r="G28" s="15" t="n"/>
       <c r="H28" s="15" t="n"/>
-      <c r="I28" s="16" t="n"/>
+      <c r="I28" s="15" t="n"/>
+      <c r="J28" s="15" t="n"/>
+      <c r="K28" s="15" t="n"/>
+      <c r="L28" s="16" t="n"/>
     </row>
     <row r="29" ht="32" customHeight="1">
       <c r="B29" s="5" t="n">
@@ -4683,12 +5511,15 @@
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr"/>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr"/>
+      <c r="I29" s="6" t="inlineStr"/>
+      <c r="J29" s="6" t="inlineStr"/>
+      <c r="K29" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I29" s="6" t="inlineStr"/>
+      <c r="L29" s="6" t="inlineStr"/>
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="B30" s="5" t="n">
@@ -4714,13 +5545,24 @@
           <t>Attendu : un tableau des écarts avec explication. Alerte : écarts non suivis.</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr"/>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Suivi des écarts chaque mois.</t>
+        </is>
+      </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
+          <t>Écart = cotisations attendues − cotisations reçues</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr"/>
+      <c r="J30" s="6" t="inlineStr"/>
+      <c r="K30" s="6" t="inlineStr">
+        <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr"/>
+      <c r="L30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="B31" s="14" t="inlineStr">
@@ -4734,7 +5576,10 @@
       <c r="F31" s="15" t="n"/>
       <c r="G31" s="15" t="n"/>
       <c r="H31" s="15" t="n"/>
-      <c r="I31" s="16" t="n"/>
+      <c r="I31" s="15" t="n"/>
+      <c r="J31" s="15" t="n"/>
+      <c r="K31" s="15" t="n"/>
+      <c r="L31" s="16" t="n"/>
     </row>
     <row r="32" ht="32" customHeight="1">
       <c r="B32" s="5" t="n">
@@ -4761,12 +5606,15 @@
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr"/>
-      <c r="H32" s="17" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr"/>
+      <c r="I32" s="6" t="inlineStr"/>
+      <c r="J32" s="6" t="inlineStr"/>
+      <c r="K32" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I32" s="6" t="inlineStr"/>
+      <c r="L32" s="6" t="inlineStr"/>
     </row>
     <row r="33" ht="46" customHeight="1">
       <c r="B33" s="5" t="n">
@@ -4794,15 +5642,26 @@
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
+          <t>Projection des départs à la retraite.</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>Année de départ = année de naissance + âge de retraite</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr"/>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
           <t>Texte de référence</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="K33" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I33" s="6" t="inlineStr"/>
+      <c r="L33" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="B35" s="2" t="inlineStr">
@@ -4841,21 +5700,21 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="B39:I39"/>
-    <mergeCell ref="B25:I25"/>
-    <mergeCell ref="B38:I38"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B36:I36"/>
-    <mergeCell ref="B37:I37"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="B4:L4"/>
+    <mergeCell ref="B13:L13"/>
+    <mergeCell ref="B38:L38"/>
+    <mergeCell ref="B39:L39"/>
+    <mergeCell ref="B25:L25"/>
+    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="B37:L37"/>
+    <mergeCell ref="B28:L28"/>
+    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="B31:L31"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="B8:L8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H8:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K8:K34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4871,18 +5730,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I30"/>
+  <dimension ref="B2:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -4909,7 +5771,7 @@
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usage interne : les colonnes « À quoi elle sert » et « Explication » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
+          <t>Usage interne : les colonnes marquées « interne » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
         </is>
       </c>
     </row>
@@ -4941,15 +5803,30 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
+          <t>Méthodes possibles (interne)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Formule (interne)</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Source et argument (interne)</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
           <t>Document à demander</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Réponse obtenue</t>
         </is>
@@ -4967,9 +5844,12 @@
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
       <c r="H8" s="15" t="n"/>
-      <c r="I8" s="16" t="n"/>
-    </row>
-    <row r="9" ht="32" customHeight="1">
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="16" t="n"/>
+    </row>
+    <row r="9" ht="46" customHeight="1">
       <c r="B9" s="5" t="n">
         <v>1</v>
       </c>
@@ -4994,14 +5874,17 @@
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr"/>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
+      <c r="L9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="46" customHeight="1">
       <c r="B10" s="5" t="n">
         <v>2</v>
       </c>
@@ -5025,17 +5908,20 @@
           <t>Extraction = export des données vers Excel. Attendu : oui, ou seulement la situation actuelle.</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>Extractions Excel</t>
         </is>
       </c>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="K10" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="B11" s="5" t="n">
@@ -5061,13 +5947,24 @@
           <t>Historique = données passées conservées. Écrasé = l'ancienne version disparaît. Si écrasé, les années passées sont à reconstituer.</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr"/>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Si écrasé : reconstitution avec les mouvements datés.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Effectif fin = effectif début + entrées − sorties</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="B12" s="5" t="n">
@@ -5094,12 +5991,15 @@
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="B13" s="5" t="n">
@@ -5126,12 +6026,15 @@
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr"/>
-      <c r="H13" s="17" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr"/>
+      <c r="K13" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="B14" s="14" t="inlineStr">
@@ -5145,7 +6048,10 @@
       <c r="F14" s="15" t="n"/>
       <c r="G14" s="15" t="n"/>
       <c r="H14" s="15" t="n"/>
-      <c r="I14" s="16" t="n"/>
+      <c r="I14" s="15" t="n"/>
+      <c r="J14" s="15" t="n"/>
+      <c r="K14" s="15" t="n"/>
+      <c r="L14" s="16" t="n"/>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="B15" s="5" t="n">
@@ -5172,14 +6078,21 @@
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr"/>
-      <c r="H15" s="17" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Offre technique p. 25 : situation au 31/08/2026 à produire par le FPPN.</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr"/>
-    </row>
-    <row r="16" ht="46" customHeight="1">
+      <c r="L15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
       <c r="B16" s="5" t="n">
         <v>7</v>
       </c>
@@ -5204,14 +6117,21 @@
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr"/>
-      <c r="H16" s="17" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>Règlement 03/2012/CM/UEMOA (PCMS) ; SYSCOHADA révisé depuis 2018.</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr"/>
+      <c r="K16" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr"/>
-    </row>
-    <row r="17" ht="32" customHeight="1">
+      <c r="L16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17" ht="46" customHeight="1">
       <c r="B17" s="5" t="n">
         <v>8</v>
       </c>
@@ -5236,12 +6156,19 @@
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr"/>
-      <c r="H17" s="17" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>ISA 540 révisée (exercices ouverts dès le 15/12/2019) : méthode et hypothèses à justifier.</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr"/>
+      <c r="K17" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr"/>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="B18" s="5" t="n">
@@ -5268,12 +6195,15 @@
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr"/>
-      <c r="H18" s="17" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr"/>
+      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr"/>
+      <c r="K18" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr"/>
+      <c r="L18" s="6" t="inlineStr"/>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="B19" s="5" t="n">
@@ -5299,19 +6229,22 @@
           <t>Attendu : un budget annuel, plus rarement sur plusieurs années.</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="6" t="inlineStr"/>
+      <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>Budgets et prévisions</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20" ht="32" customHeight="1">
+      <c r="L19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20" ht="46" customHeight="1">
       <c r="B20" s="5" t="n">
         <v>11</v>
       </c>
@@ -5335,13 +6268,24 @@
           <t>Frais de gestion = coûts de fonctionnement. Attendu : souvent un total global, sans détail par activité.</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Frais répartis par activité (effectifs, temps passé).</t>
+        </is>
+      </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
+          <t>Taux de frais = frais ÷ cotisations</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr"/>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="B21" s="14" t="inlineStr">
@@ -5355,7 +6299,10 @@
       <c r="F21" s="15" t="n"/>
       <c r="G21" s="15" t="n"/>
       <c r="H21" s="15" t="n"/>
-      <c r="I21" s="16" t="n"/>
+      <c r="I21" s="15" t="n"/>
+      <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
+      <c r="L21" s="16" t="n"/>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="B22" s="5" t="n">
@@ -5381,19 +6328,26 @@
           <t>Attendu : statuts datés et versions successives. Alerte : textes jugés caducs lors d'une AG extraordinaire.</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr"/>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>Règlement 07/2009/CM/UEMOA : les statuts fixent les modalités des cotisations.</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>Statuts et règlements successifs</t>
         </is>
       </c>
-      <c r="H22" s="17" t="inlineStr">
+      <c r="K22" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="32" customHeight="1">
+      <c r="L22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="46" customHeight="1">
       <c r="B23" s="5" t="n">
         <v>13</v>
       </c>
@@ -5419,17 +6373,32 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
+          <t>Provision si la perte est probable et chiffrable.</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>Provision = meilleure estimation de la somme à payer</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>Principe de prudence (SYSCOHADA révisé depuis 2018 ; PCMS) : un risque probable donne lieu à provision.</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
           <t>État des litiges</t>
         </is>
       </c>
-      <c r="H23" s="17" t="inlineStr">
+      <c r="K23" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I23" s="6" t="inlineStr"/>
-    </row>
-    <row r="24" ht="32" customHeight="1">
+      <c r="L23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24" ht="46" customHeight="1">
       <c r="B24" s="5" t="n">
         <v>14</v>
       </c>
@@ -5453,17 +6422,24 @@
           <t>Agrément = autorisation de fonctionner délivrée par l'AIRMS. Attendu : oui, avec un numéro.</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>Règlement 07/2009/CM/UEMOA : agrément et immatriculation par l'organe national (AIRMS en Côte d'Ivoire).</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>Agrément et courriers de l'AIRMS</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr"/>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="B25" s="5" t="n">
@@ -5489,19 +6465,22 @@
           <t>CGRAE = caisse de retraite des fonctionnaires. Attendu : une convention signée et datée.</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr"/>
+      <c r="H25" s="6" t="inlineStr"/>
+      <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="6" t="inlineStr">
         <is>
           <t>Convention CGRAE</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="K25" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26" ht="32" customHeight="1">
+      <c r="L25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26" ht="46" customHeight="1">
       <c r="B26" s="5" t="n">
         <v>16</v>
       </c>
@@ -5526,12 +6505,15 @@
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr"/>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr"/>
+      <c r="I26" s="6" t="inlineStr"/>
+      <c r="J26" s="6" t="inlineStr"/>
+      <c r="K26" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="B27" s="14" t="inlineStr">
@@ -5545,9 +6527,12 @@
       <c r="F27" s="15" t="n"/>
       <c r="G27" s="15" t="n"/>
       <c r="H27" s="15" t="n"/>
-      <c r="I27" s="16" t="n"/>
-    </row>
-    <row r="28" ht="32" customHeight="1">
+      <c r="I27" s="15" t="n"/>
+      <c r="J27" s="15" t="n"/>
+      <c r="K27" s="15" t="n"/>
+      <c r="L27" s="16" t="n"/>
+    </row>
+    <row r="28" ht="46" customHeight="1">
       <c r="B28" s="5" t="n">
         <v>17</v>
       </c>
@@ -5571,17 +6556,20 @@
           <t>Inventaire = liste des biens avec leur valeur. Attendu : une liste, souvent sans valeur à jour.</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr"/>
+      <c r="H28" s="6" t="inlineStr"/>
+      <c r="I28" s="6" t="inlineStr"/>
+      <c r="J28" s="6" t="inlineStr">
         <is>
           <t>Inventaire immobilier</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="K28" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="B29" s="14" t="inlineStr">
@@ -5595,7 +6583,10 @@
       <c r="F29" s="15" t="n"/>
       <c r="G29" s="15" t="n"/>
       <c r="H29" s="15" t="n"/>
-      <c r="I29" s="16" t="n"/>
+      <c r="I29" s="15" t="n"/>
+      <c r="J29" s="15" t="n"/>
+      <c r="K29" s="15" t="n"/>
+      <c r="L29" s="16" t="n"/>
     </row>
     <row r="30" ht="46" customHeight="1">
       <c r="B30" s="5" t="n">
@@ -5621,30 +6612,33 @@
           <t>Attendu : des rapports avec constats. Note ceux qui touchent tes sujets.</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr"/>
+      <c r="H30" s="6" t="inlineStr"/>
+      <c r="I30" s="6" t="inlineStr"/>
+      <c r="J30" s="6" t="inlineStr">
         <is>
           <t>Rapports d'audit interne</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="K30" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr"/>
+      <c r="L30" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B4:L4"/>
+    <mergeCell ref="B21:L21"/>
+    <mergeCell ref="B29:L29"/>
+    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="B14:L14"/>
+    <mergeCell ref="B27:L27"/>
+    <mergeCell ref="B8:L8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H8:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K8:K31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5660,19 +6654,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:J26"/>
+  <dimension ref="B2:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -5699,7 +6696,7 @@
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Usage interne : les colonnes « À quoi elle sert » et « Explication » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
+          <t>Usage interne : les colonnes marquées « interne » sont réservées à l'équipe Adenka. Ne pas transmettre ce fichier au client.</t>
         </is>
       </c>
     </row>
@@ -5731,20 +6728,35 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
+          <t>Méthodes possibles (interne)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Formule (interne)</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Source et argument (interne)</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
           <t>Document à demander</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Interlocuteur supposé</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -5763,7 +6775,10 @@
       <c r="G8" s="15" t="n"/>
       <c r="H8" s="15" t="n"/>
       <c r="I8" s="15" t="n"/>
-      <c r="J8" s="16" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="15" t="n"/>
+      <c r="M8" s="16" t="n"/>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="B9" s="5" t="n">
@@ -5791,20 +6806,31 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
+          <t>Encours et impayés par emprunteur.</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Taux d'impayés = impayés ÷ encours</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
           <t>Encours par emprunteur</t>
         </is>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="K9" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr">
         <is>
           <t>Directeur du Grenier du Policier ; Caisse de crédit mutuel (rattachée au DGA)</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="B10" s="5" t="n">
@@ -5832,20 +6858,35 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
+          <t>Dépréciation par tranche d'ancienneté des impayés.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Dépréciation = impayés × taux de la tranche</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Principe de prudence (SYSCOHADA révisé depuis 2018 ; PCMS) : un prêt douteux est déprécié.</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
           <t>Échéancier et impayés</t>
         </is>
       </c>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="K10" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr">
         <is>
           <t>Directeur du Grenier du Policier</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr"/>
+      <c r="M10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="B11" s="5" t="n">
@@ -5873,20 +6914,31 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
+          <t>Projection des remboursements futurs.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Échéance constante = capital × i ÷ (1 − (1+i)^−n)</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
           <t>Conditions des prêts</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>Directeur du Grenier du Policier</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr"/>
+      <c r="M11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="B12" s="14" t="inlineStr">
@@ -5901,7 +6953,10 @@
       <c r="G12" s="15" t="n"/>
       <c r="H12" s="15" t="n"/>
       <c r="I12" s="15" t="n"/>
-      <c r="J12" s="16" t="n"/>
+      <c r="J12" s="15" t="n"/>
+      <c r="K12" s="15" t="n"/>
+      <c r="L12" s="15" t="n"/>
+      <c r="M12" s="16" t="n"/>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="B13" s="5" t="n">
@@ -5927,22 +6982,25 @@
           <t>Allocation = somme versée lors d'un événement (décès, naissance, mariage). Attendu : une liste et des montants.</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>Barèmes des aides</t>
         </is>
       </c>
-      <c r="H13" s="17" t="inlineStr">
+      <c r="K13" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>Chef du service des affaires sociales</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr"/>
+      <c r="M13" s="6" t="inlineStr"/>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="B14" s="5" t="n">
@@ -5970,20 +7028,31 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
+          <t>Coût moyen par bénéficiaire.</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Coût moyen = prestations santé ÷ nombre de bénéficiaires</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
           <t>Statistiques des soins</t>
         </is>
       </c>
-      <c r="H14" s="17" t="inlineStr">
+      <c r="K14" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="L14" s="6" t="inlineStr">
         <is>
           <t>Chef du service médical</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr"/>
+      <c r="M14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="B15" s="5" t="n">
@@ -6009,22 +7078,25 @@
           <t>Attendu : facture interne ou budget global. Sert à isoler le coût réel des soins.</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Comptes du centre médical</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>Responsable du CM-FPPN</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr"/>
+      <c r="M15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="B16" s="14" t="inlineStr">
@@ -6039,9 +7111,12 @@
       <c r="G16" s="15" t="n"/>
       <c r="H16" s="15" t="n"/>
       <c r="I16" s="15" t="n"/>
-      <c r="J16" s="16" t="n"/>
-    </row>
-    <row r="17" ht="46" customHeight="1">
+      <c r="J16" s="15" t="n"/>
+      <c r="K16" s="15" t="n"/>
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="16" t="n"/>
+    </row>
+    <row r="17" ht="60" customHeight="1">
       <c r="B17" s="5" t="n">
         <v>7</v>
       </c>
@@ -6067,20 +7142,31 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
+          <t>Contrôle des comptes individuels.</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Solde fin = solde début + versements + intérêts − retraits</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
           <t>Comptes individuels d'épargne</t>
         </is>
       </c>
-      <c r="H17" s="17" t="inlineStr">
+      <c r="K17" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>Gestionnaire de l'épargne (poste absent de l'organigramme ; probablement service comptabilité)</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr"/>
+      <c r="M17" s="6" t="inlineStr"/>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="B18" s="5" t="n">
@@ -6108,20 +7194,31 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
+          <t>Projection des paiements de fin de carrière.</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Paiement prévu = Σ soldes des mutualistes qui partent cette année</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
           <t>État des paiements d'épargne</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="K18" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr">
+      <c r="L18" s="6" t="inlineStr">
         <is>
           <t>Gestionnaire de l'épargne</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr"/>
+      <c r="M18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="B19" s="14" t="inlineStr">
@@ -6136,7 +7233,10 @@
       <c r="G19" s="15" t="n"/>
       <c r="H19" s="15" t="n"/>
       <c r="I19" s="15" t="n"/>
-      <c r="J19" s="16" t="n"/>
+      <c r="J19" s="15" t="n"/>
+      <c r="K19" s="15" t="n"/>
+      <c r="L19" s="15" t="n"/>
+      <c r="M19" s="16" t="n"/>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="B20" s="5" t="n">
@@ -6164,20 +7264,31 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
+          <t>Valeur d'expertise récente.</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>Code CIMA art. 335-12 : principes d'évaluation des placements. Référence technique.</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
           <t>Évaluations et revenus</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>Responsable patrimoine et projets immobiliers (rattaché au service juridique)</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr"/>
+      <c r="M20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="B21" s="14" t="inlineStr">
@@ -6192,7 +7303,10 @@
       <c r="G21" s="15" t="n"/>
       <c r="H21" s="15" t="n"/>
       <c r="I21" s="15" t="n"/>
-      <c r="J21" s="16" t="n"/>
+      <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
+      <c r="L21" s="15" t="n"/>
+      <c r="M21" s="16" t="n"/>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="B22" s="5" t="n">
@@ -6218,22 +7332,25 @@
           <t>PV = procès-verbal, compte rendu officiel d'une réunion. Attendu : une liste des décisions avec leurs dates.</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr"/>
+      <c r="I22" s="6" t="inlineStr"/>
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>Procès-verbaux et décisions</t>
         </is>
       </c>
-      <c r="H22" s="17" t="inlineStr">
+      <c r="K22" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr">
+      <c r="L22" s="6" t="inlineStr">
         <is>
           <t>Chef de cabinet ; secrétariat de direction</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr"/>
+      <c r="M22" s="6" t="inlineStr"/>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="B23" s="5" t="n">
@@ -6259,22 +7376,25 @@
           <t>Attendu : études internes ou de cabinets. Demande les copies.</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr"/>
+      <c r="H23" s="6" t="inlineStr"/>
+      <c r="I23" s="6" t="inlineStr"/>
+      <c r="J23" s="6" t="inlineStr">
         <is>
           <t>Études existantes</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="K23" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I23" s="6" t="inlineStr">
+      <c r="L23" s="6" t="inlineStr">
         <is>
           <t>Conseillers techniques du DG</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr"/>
+      <c r="M23" s="6" t="inlineStr"/>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="B24" s="5" t="n">
@@ -6300,22 +7420,29 @@
           <t>Attendu : courriers, rapports de contrôle, injonctions.</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>Décision UEMOA n°05/2022 : indicateurs et ratios prudentiels des mutuelles.</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>Courriers de l'AIRMS</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr">
+      <c r="L24" s="6" t="inlineStr">
         <is>
           <t>Directeur général ; chef de cabinet</t>
         </is>
       </c>
-      <c r="J24" s="6" t="inlineStr"/>
+      <c r="M24" s="6" t="inlineStr"/>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="B25" s="5" t="n">
@@ -6343,20 +7470,27 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
+          <t>Hypothèse d'âge de départ utilisée dans la projection.</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr"/>
+      <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
           <t>Texte de référence</t>
         </is>
       </c>
-      <c r="H25" s="17" t="inlineStr">
+      <c r="K25" s="17" t="inlineStr">
         <is>
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr">
+      <c r="L25" s="6" t="inlineStr">
         <is>
           <t>Service du personnel du FPPN ; à défaut, DRH de la Police nationale</t>
         </is>
       </c>
-      <c r="J25" s="6" t="inlineStr"/>
+      <c r="M25" s="6" t="inlineStr"/>
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="B26" s="5" t="n">
@@ -6384,33 +7518,48 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
+          <t>Comparer la mortalité observée à la table CIMA H.</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Taux de décès = décès de l'année ÷ effectif exposé</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>Code CIMA art. 338 : table CIMA H pour le décès. Référence technique.</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
           <t>Statistiques</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="K26" s="6" t="inlineStr">
         <is>
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
+      <c r="L26" s="6" t="inlineStr">
         <is>
           <t>Service des affaires sociales ; DRH de la Police nationale</t>
         </is>
       </c>
-      <c r="J26" s="6" t="inlineStr"/>
+      <c r="M26" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B5:J5"/>
-    <mergeCell ref="B19:J19"/>
-    <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B4:J4"/>
-    <mergeCell ref="B12:J12"/>
-    <mergeCell ref="B21:J21"/>
-    <mergeCell ref="B16:J16"/>
+    <mergeCell ref="B16:M16"/>
+    <mergeCell ref="B5:M5"/>
+    <mergeCell ref="B19:M19"/>
+    <mergeCell ref="B21:M21"/>
+    <mergeCell ref="B8:M8"/>
+    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="B12:M12"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H8:H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K8:K27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Entretien sinistres et prestations : CR, note interne, demande complémentaire, plan et script d'analyses
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_Guides_entretiens_actuariat_20261016.xlsx
+++ b/FPPN_Guides_entretiens_actuariat_20261016.xlsx
@@ -1075,7 +1075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:L44"/>
+  <dimension ref="B1:S44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1092,6 +1092,7 @@
     <col width="30" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1120,6 +1121,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1231,7 +1233,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>Régime obligatoire : maladie, maternité, décès, invalidité. Décès du policier : capital + frais funéraires (300 000 FCFA depuis 2023). Décès du conjoint ou d'un enfant : montants par corps. Allocation d'accouchement 100 000 FCFA (si grossesse non suivie par le fonds). Autres : produit retraite (mai 2007), flotte automobile.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="B10" s="5" t="n">
@@ -1274,7 +1280,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>Capital par corps (ancien barème) : 2 M commissaires, 1 M sous-officiers, officiers à confirmer. Ex. ayants droit officier (ancien tableau) : épouse 700 000, enfant 150 000 (à confirmer). 2013-2015 : 15 × salaire de base ; 2015-2020 : 13 × salaire de base.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="B11" s="5" t="n">
@@ -1313,7 +1323,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>Oui : 2001-11/2013 forfait par corps (interne) ; 11/2013-2015 externalisé, 15 × salaire de base ; 2015-2020 externalisé, 13 × salaire de base + barème frais funéraires par grade (1 M à 3 M puis 4 M) ; 2021-2023 retour au forfait par corps, frais funéraires supprimés ; depuis 2023 frais funéraires 300 000 FCFA ; 2026 revalorisation à l'étude (3 options).</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="B12" s="5" t="n">
@@ -1360,7 +1374,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L12" s="6" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>En une fois. Réparti entre les héritiers selon les documents de justice (succession). Mineurs : paiement à l'administrateur légal.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="B13" s="5" t="n">
@@ -1407,7 +1425,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>Oui pour la maladie uniquement, à condition de se réinscrire après le départ (sinon sortie du fichier).</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="B14" s="5" t="n">
@@ -1446,7 +1468,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>Réponse floue : « les retraités ne sont pas pris en compte avec [la CGRAE], c'est uniquement la maladie ». À clarifier.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="B15" s="5" t="n">
@@ -1481,7 +1507,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>Carence au lancement du fonds uniquement. Aujourd'hui, affiliation automatique dès l'entrée dans la police.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="14" t="inlineStr">
@@ -1537,7 +1567,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>1. Courrier du chef hiérarchique (OPJ). 2. La famille reçoit la liste des pièces. 3. Agent déclaration enregistre, agent traitement traite. 4. Chef de service vérifie, met à jour son tableau de bord, signe. 5. Paiement par la comptabilité (programmation). Dossiers assureurs signés par le DG.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="B18" s="5" t="n">
@@ -1580,7 +1614,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr"/>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>Pas de délai chiffré. Le délai vient surtout des familles (documents de justice). Traitement interne rapide (le jour même selon lui). Paiement sur programmation, moins d'un mois.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="B19" s="5" t="n">
@@ -1627,7 +1665,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr"/>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>Pas de délai cité. Dossiers anciens encore ouverts (depuis 2004) à cause de litiges familiaux.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="B20" s="5" t="n">
@@ -1678,7 +1720,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>Pas de chiffre. Sinistres antérieurs à 2013 non payés. Sinistres 2022 à 2026 mélangés, tri demandé pour 2026. Simulation : sinistralité 113 % en juin 2026.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="B21" s="5" t="n">
@@ -1713,7 +1759,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L21" s="6" t="inlineStr"/>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>Oui avant 2013 (fonds décès mélangé avec les autres prestations), motif de l'externalisation de 2013.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="B22" s="5" t="n">
@@ -1764,7 +1814,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L22" s="6" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>Non abordé précisément. Service non associé aux provisions.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="14" t="inlineStr">
@@ -1820,7 +1874,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>Prise en charge signée par le médecin, factures des prestataires directement à la comptabilité (tiers payant).</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="B25" s="5" t="n">
@@ -1863,7 +1921,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L25" s="6" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>Non précisé.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="46" customHeight="1">
       <c r="B26" s="5" t="n">
@@ -1898,7 +1960,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L26" s="6" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr">
+        <is>
+          <t>Non abordé.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="14" t="inlineStr">
@@ -1950,7 +2016,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L28" s="6" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>Pas de logiciel dédié. Tableau de bord personnel du chef de service. Logiciel en projet avec l'informaticien.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="46" customHeight="1">
       <c r="B29" s="5" t="n">
@@ -2001,7 +2071,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L29" s="6" t="inlineStr"/>
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>Oui, fichiers de sinistralité 2019-2026 promis. Base demandée au format modèle (demande n°28).</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="46" customHeight="1">
       <c r="B30" s="5" t="n">
@@ -2036,7 +2110,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L30" s="6" t="inlineStr"/>
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>Non vérifié.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="46" customHeight="1">
       <c r="B31" s="5" t="n">
@@ -2083,7 +2161,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L31" s="6" t="inlineStr"/>
+      <c r="L31" s="6" t="inlineStr">
+        <is>
+          <t>Oui, tableau de bord de sinistralité. Chiffres cités : 75-76 % en 2019, 21 % en 2021, 113 % en juin 2026. Jusqu'à 125 décès par an en période de pic.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="14" t="inlineStr">
@@ -2135,7 +2217,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L33" s="6" t="inlineStr"/>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>Chef de service (signature). Proposition récente d'une validation par le directeur ou le DG. Pas de contrôle intermédiaire à la comptabilité décrit.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="46" customHeight="1">
       <c r="B34" s="5" t="n">
@@ -2170,7 +2256,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L34" s="6" t="inlineStr"/>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>Vérification des pièces (documents de justice, état civil). Volet médical : aucun contrôle (anciennes cartes, ayants droit non éligibles).</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="32" customHeight="1">
       <c r="B35" s="5" t="n">
@@ -2205,7 +2295,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L35" s="6" t="inlineStr"/>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>Non précisé.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="14" t="inlineStr">
@@ -2273,7 +2367,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L37" s="6" t="inlineStr"/>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>Litiges surtout entre membres des familles. Litiges FPPN-familles peu fréquents (courrier de rejet motivé). Litiges sur le dossier immobilier côté juridique.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="60" customHeight="1">
       <c r="B38" s="5" t="n">
@@ -2308,8 +2406,13 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L38" s="6" t="inlineStr"/>
-    </row>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>Le service n'est pas associé au provisionnement. Selon lui, les provisions ne sont pas reportées d'une année à l'autre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
     <row r="40">
       <c r="B40" s="2" t="inlineStr">
         <is>

</xml_diff>